<commit_message>
feat: Update Jupyter notebooks with execution counts and outputs
- Updated session11.ipynb to include execution counts and outputs for code cells.
- Added error handling for UnicodeDecodeError when reading encoding.txt.
- Enhanced output for reading from encoding.txt and added a new pickle file for person data.
- Updated session12.ipynb with execution counts, outputs, and improved markdown formatting.
- Added new encoding.txt file with example content.
- Added new person.pickle file with serialized Person object.
</commit_message>
<xml_diff>
--- a/ML-Excercises/Excels/Lecture_Machine_Learning_for_Natural_Language_Understanding/03-ML4NLU-Linear-Layer.xlsx
+++ b/ML-Excercises/Excels/Lecture_Machine_Learning_for_Natural_Language_Understanding/03-ML4NLU-Linear-Layer.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28025"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10125"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://o365coloradoedu-my.sharepoint.com/personal/peye9704_colorado_edu/Documents/2024/AIbyHand/spreadsheets/github/ai-by-hand-excel/workbook/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hd/Desktop/Machine Learning/ML-Excercises/Excels/Lecture_Machine_Learning_for_Natural_Language_Understanding/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="18" documentId="13_ncr:1_{038C559F-B59A-1D47-B534-25B9ECBECE90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{37381BC6-483C-49A9-BC7A-8C7D1DE1E655}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D435754-4776-A547-AC2C-620E4F6818F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13875" xr2:uid="{045A32B7-7D49-AA41-9BCB-690BF8CB81ED}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" xr2:uid="{045A32B7-7D49-AA41-9BCB-690BF8CB81ED}"/>
   </bookViews>
   <sheets>
     <sheet name="Exrcise 1-5" sheetId="1" r:id="rId1"/>
@@ -744,7 +744,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="89">
+  <cellXfs count="88">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -911,10 +911,48 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -923,19 +961,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" readingOrder="1"/>
@@ -946,33 +971,7 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -40270,42 +40269,40 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AC779A4B-5D45-B242-BD82-6967E251B652}">
   <dimension ref="A1:AI20"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.5"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="11" style="63"/>
-    <col min="2" max="2" width="4.8125" style="63" customWidth="1"/>
-    <col min="3" max="4" width="5.1875" style="63" customWidth="1"/>
-    <col min="5" max="6" width="4.6875" style="63" customWidth="1"/>
-    <col min="7" max="7" width="4" style="63" customWidth="1"/>
-    <col min="8" max="8" width="9.6875" style="63" customWidth="1"/>
-    <col min="9" max="9" width="5" style="63" customWidth="1"/>
-    <col min="10" max="10" width="4.8125" style="63" customWidth="1"/>
-    <col min="11" max="11" width="5.3125" style="63" customWidth="1"/>
-    <col min="12" max="12" width="4.6875" style="63" customWidth="1"/>
-    <col min="13" max="13" width="4.5" style="63" customWidth="1"/>
-    <col min="14" max="14" width="4.8125" style="63" customWidth="1"/>
-    <col min="15" max="15" width="9.3125" style="63" customWidth="1"/>
-    <col min="16" max="17" width="4.8125" style="63" customWidth="1"/>
-    <col min="18" max="18" width="5.3125" style="63" customWidth="1"/>
-    <col min="19" max="19" width="4.5" style="63" customWidth="1"/>
-    <col min="20" max="20" width="4.6875" style="63" customWidth="1"/>
-    <col min="21" max="21" width="4.8125" style="63" customWidth="1"/>
-    <col min="22" max="22" width="9.3125" style="63" customWidth="1"/>
-    <col min="23" max="24" width="4.3125" style="63" customWidth="1"/>
-    <col min="25" max="25" width="4.6875" style="63" customWidth="1"/>
-    <col min="26" max="26" width="4.3125" style="63" customWidth="1"/>
-    <col min="27" max="27" width="4.5" style="63" customWidth="1"/>
-    <col min="28" max="28" width="4.3125" style="63" customWidth="1"/>
-    <col min="29" max="29" width="10" style="63" customWidth="1"/>
-    <col min="30" max="30" width="4.6875" style="63" customWidth="1"/>
-    <col min="31" max="31" width="5.3125" style="63" customWidth="1"/>
-    <col min="32" max="32" width="5.1875" style="63" customWidth="1"/>
-    <col min="33" max="34" width="5" style="63" customWidth="1"/>
-    <col min="35" max="35" width="4.6875" style="63" customWidth="1"/>
-    <col min="36" max="16384" width="11" style="63"/>
+    <col min="2" max="2" width="4.83203125" customWidth="1"/>
+    <col min="3" max="4" width="5.1640625" customWidth="1"/>
+    <col min="5" max="6" width="4.6640625" customWidth="1"/>
+    <col min="7" max="7" width="4" customWidth="1"/>
+    <col min="8" max="8" width="9.6640625" customWidth="1"/>
+    <col min="9" max="9" width="5" customWidth="1"/>
+    <col min="10" max="10" width="4.83203125" customWidth="1"/>
+    <col min="11" max="11" width="5.33203125" customWidth="1"/>
+    <col min="12" max="12" width="4.6640625" customWidth="1"/>
+    <col min="13" max="13" width="4.5" customWidth="1"/>
+    <col min="14" max="14" width="4.83203125" customWidth="1"/>
+    <col min="15" max="15" width="9.33203125" customWidth="1"/>
+    <col min="16" max="17" width="4.83203125" customWidth="1"/>
+    <col min="18" max="18" width="5.33203125" customWidth="1"/>
+    <col min="19" max="19" width="4.5" customWidth="1"/>
+    <col min="20" max="20" width="4.6640625" customWidth="1"/>
+    <col min="21" max="21" width="4.83203125" customWidth="1"/>
+    <col min="22" max="22" width="9.33203125" customWidth="1"/>
+    <col min="23" max="24" width="4.33203125" customWidth="1"/>
+    <col min="25" max="25" width="4.6640625" customWidth="1"/>
+    <col min="26" max="26" width="4.33203125" customWidth="1"/>
+    <col min="27" max="27" width="4.5" customWidth="1"/>
+    <col min="28" max="28" width="4.33203125" customWidth="1"/>
+    <col min="29" max="29" width="10" customWidth="1"/>
+    <col min="30" max="30" width="4.6640625" customWidth="1"/>
+    <col min="31" max="31" width="5.33203125" customWidth="1"/>
+    <col min="32" max="32" width="5.1640625" customWidth="1"/>
+    <col min="33" max="34" width="5" customWidth="1"/>
+    <col min="35" max="35" width="4.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" s="2" customFormat="1" ht="19.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:35" s="2" customFormat="1" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>44</v>
       </c>
@@ -40323,7 +40320,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="2" spans="1:35" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.55000000000000004">
+    <row r="2" spans="1:35" s="2" customFormat="1" ht="19" x14ac:dyDescent="0.25">
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -40332,11 +40329,11 @@
       <c r="J2" s="1"/>
       <c r="O2" s="1"/>
     </row>
-    <row r="3" spans="1:35" ht="18.399999999999999" thickBot="1" x14ac:dyDescent="0.6">
+    <row r="3" spans="1:35" ht="20" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2"/>
       <c r="B3" s="2" t="str">
         <f>IF(ISBLANK(F9)=TRUE,"NOT DONE",IF(B5=F9,"CORRECT", "INCORRECT"))</f>
-        <v>NOT DONE</v>
+        <v>CORRECT</v>
       </c>
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
@@ -40344,7 +40341,7 @@
       <c r="F3" s="2"/>
       <c r="I3" s="2" t="str">
         <f>IF(ISBLANK(M9)=TRUE,"NOT DONE",IF(I5=M9,"CORRECT", "INCORRECT"))</f>
-        <v>NOT DONE</v>
+        <v>CORRECT</v>
       </c>
       <c r="J3" s="2"/>
       <c r="K3" s="2"/>
@@ -40352,7 +40349,7 @@
       <c r="M3" s="2"/>
       <c r="P3" s="2" t="str">
         <f>IF(ISBLANK(T9)=TRUE,"NOT DONE",IF(P5=T9,"CORRECT", "INCORRECT"))</f>
-        <v>NOT DONE</v>
+        <v>CORRECT</v>
       </c>
       <c r="Q3" s="2"/>
       <c r="R3" s="2"/>
@@ -40360,7 +40357,7 @@
       <c r="T3" s="2"/>
       <c r="W3" s="2" t="str">
         <f>IF(ISBLANK(AA10)=TRUE,"NOT DONE",IF(W5=AA10,"CORRECT", "INCORRECT"))</f>
-        <v>NOT DONE</v>
+        <v>CORRECT</v>
       </c>
       <c r="X3" s="2"/>
       <c r="Y3" s="2"/>
@@ -40368,57 +40365,57 @@
       <c r="AA3" s="2"/>
       <c r="AD3" s="2" t="str">
         <f>IF(ISBLANK(AH11)=TRUE,"NOT DONE",IF(AD5=AH11,"CORRECT", "INCORRECT"))</f>
-        <v>NOT DONE</v>
+        <v>CORRECT</v>
       </c>
       <c r="AE3" s="2"/>
       <c r="AF3" s="2"/>
       <c r="AG3" s="2"/>
       <c r="AH3" s="2"/>
     </row>
-    <row r="4" spans="1:35" ht="19.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="4" spans="1:35" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2"/>
-      <c r="B4" s="64" t="s">
+      <c r="B4" s="80" t="s">
         <v>0</v>
       </c>
-      <c r="C4" s="65"/>
-      <c r="D4" s="65"/>
-      <c r="E4" s="65"/>
-      <c r="F4" s="65"/>
-      <c r="G4" s="66"/>
-      <c r="I4" s="64" t="s">
+      <c r="C4" s="81"/>
+      <c r="D4" s="81"/>
+      <c r="E4" s="81"/>
+      <c r="F4" s="81"/>
+      <c r="G4" s="82"/>
+      <c r="I4" s="80" t="s">
         <v>1</v>
       </c>
-      <c r="J4" s="65"/>
-      <c r="K4" s="65"/>
-      <c r="L4" s="65"/>
-      <c r="M4" s="65"/>
-      <c r="N4" s="66"/>
-      <c r="P4" s="64" t="s">
+      <c r="J4" s="81"/>
+      <c r="K4" s="81"/>
+      <c r="L4" s="81"/>
+      <c r="M4" s="81"/>
+      <c r="N4" s="82"/>
+      <c r="P4" s="80" t="s">
         <v>2</v>
       </c>
-      <c r="Q4" s="65"/>
-      <c r="R4" s="65"/>
-      <c r="S4" s="65"/>
-      <c r="T4" s="65"/>
-      <c r="U4" s="66"/>
-      <c r="W4" s="64" t="s">
+      <c r="Q4" s="81"/>
+      <c r="R4" s="81"/>
+      <c r="S4" s="81"/>
+      <c r="T4" s="81"/>
+      <c r="U4" s="82"/>
+      <c r="W4" s="80" t="s">
         <v>3</v>
       </c>
-      <c r="X4" s="65"/>
-      <c r="Y4" s="65"/>
-      <c r="Z4" s="65"/>
-      <c r="AA4" s="65"/>
-      <c r="AB4" s="66"/>
-      <c r="AD4" s="64" t="s">
+      <c r="X4" s="81"/>
+      <c r="Y4" s="81"/>
+      <c r="Z4" s="81"/>
+      <c r="AA4" s="81"/>
+      <c r="AB4" s="82"/>
+      <c r="AD4" s="80" t="s">
         <v>4</v>
       </c>
-      <c r="AE4" s="65"/>
-      <c r="AF4" s="65"/>
-      <c r="AG4" s="65"/>
-      <c r="AH4" s="65"/>
-      <c r="AI4" s="66"/>
+      <c r="AE4" s="81"/>
+      <c r="AF4" s="81"/>
+      <c r="AG4" s="81"/>
+      <c r="AH4" s="81"/>
+      <c r="AI4" s="82"/>
     </row>
-    <row r="5" spans="1:35" ht="18" x14ac:dyDescent="0.55000000000000004">
+    <row r="5" spans="1:35" ht="19" x14ac:dyDescent="0.25">
       <c r="A5" s="2"/>
       <c r="B5" s="14">
         <f>C9*F7+D9</f>
@@ -40428,7 +40425,7 @@
       <c r="D5" s="2"/>
       <c r="E5" s="2"/>
       <c r="F5" s="2"/>
-      <c r="G5" s="67"/>
+      <c r="G5" s="63"/>
       <c r="I5" s="14">
         <f>J9*M7+K9</f>
         <v>14</v>
@@ -40437,7 +40434,7 @@
       <c r="K5" s="2"/>
       <c r="L5" s="2"/>
       <c r="M5" s="2"/>
-      <c r="N5" s="67"/>
+      <c r="N5" s="63"/>
       <c r="P5" s="14">
         <f>Q9*T7+R9</f>
         <v>11</v>
@@ -40446,7 +40443,7 @@
       <c r="R5" s="2"/>
       <c r="S5" s="2"/>
       <c r="T5" s="2"/>
-      <c r="U5" s="67"/>
+      <c r="U5" s="63"/>
       <c r="W5" s="14">
         <f>AA7*X10+Y10</f>
         <v>10</v>
@@ -40455,7 +40452,7 @@
       <c r="Y5" s="2"/>
       <c r="Z5" s="2"/>
       <c r="AA5" s="2"/>
-      <c r="AB5" s="67"/>
+      <c r="AB5" s="63"/>
       <c r="AD5" s="14">
         <f>AH7*AE11+AF11</f>
         <v>2</v>
@@ -40464,9 +40461,9 @@
       <c r="AF5" s="2"/>
       <c r="AG5" s="2"/>
       <c r="AH5" s="2"/>
-      <c r="AI5" s="67"/>
+      <c r="AI5" s="63"/>
     </row>
-    <row r="6" spans="1:35" ht="19.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="6" spans="1:35" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2"/>
       <c r="B6" s="10"/>
       <c r="C6" s="1"/>
@@ -40475,7 +40472,7 @@
       <c r="F6" s="47" t="s">
         <v>46</v>
       </c>
-      <c r="G6" s="68"/>
+      <c r="G6" s="64"/>
       <c r="I6" s="10"/>
       <c r="J6" s="1"/>
       <c r="K6" s="1"/>
@@ -40483,7 +40480,7 @@
       <c r="M6" s="47" t="s">
         <v>46</v>
       </c>
-      <c r="N6" s="68"/>
+      <c r="N6" s="64"/>
       <c r="P6" s="10"/>
       <c r="Q6" s="1"/>
       <c r="R6" s="1"/>
@@ -40491,7 +40488,7 @@
       <c r="T6" s="47" t="s">
         <v>46</v>
       </c>
-      <c r="U6" s="68"/>
+      <c r="U6" s="64"/>
       <c r="W6" s="10"/>
       <c r="X6" s="1"/>
       <c r="Y6" s="1"/>
@@ -40499,7 +40496,7 @@
       <c r="AA6" s="47" t="s">
         <v>46</v>
       </c>
-      <c r="AB6" s="68"/>
+      <c r="AB6" s="64"/>
       <c r="AD6" s="10"/>
       <c r="AE6" s="1"/>
       <c r="AF6" s="1"/>
@@ -40507,9 +40504,9 @@
       <c r="AH6" s="47" t="s">
         <v>46</v>
       </c>
-      <c r="AI6" s="68"/>
+      <c r="AI6" s="64"/>
     </row>
-    <row r="7" spans="1:35" ht="18" x14ac:dyDescent="0.55000000000000004">
+    <row r="7" spans="1:35" ht="19" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="10"/>
       <c r="C7" s="1"/>
@@ -40518,7 +40515,7 @@
       <c r="F7" s="16">
         <v>4</v>
       </c>
-      <c r="G7" s="68"/>
+      <c r="G7" s="64"/>
       <c r="I7" s="10"/>
       <c r="J7" s="1"/>
       <c r="K7" s="1"/>
@@ -40526,7 +40523,7 @@
       <c r="M7" s="16">
         <v>4</v>
       </c>
-      <c r="N7" s="68"/>
+      <c r="N7" s="64"/>
       <c r="P7" s="10"/>
       <c r="Q7" s="1"/>
       <c r="R7" s="1"/>
@@ -40534,7 +40531,7 @@
       <c r="T7" s="16">
         <v>4</v>
       </c>
-      <c r="U7" s="68"/>
+      <c r="U7" s="64"/>
       <c r="W7" s="10"/>
       <c r="X7" s="1"/>
       <c r="Y7" s="1"/>
@@ -40542,7 +40539,7 @@
       <c r="AA7" s="16">
         <v>4</v>
       </c>
-      <c r="AB7" s="68"/>
+      <c r="AB7" s="64"/>
       <c r="AD7" s="10"/>
       <c r="AE7" s="1"/>
       <c r="AF7" s="1"/>
@@ -40550,9 +40547,9 @@
       <c r="AH7" s="16">
         <v>2</v>
       </c>
-      <c r="AI7" s="68"/>
+      <c r="AI7" s="64"/>
     </row>
-    <row r="8" spans="1:35" ht="19.05" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
+    <row r="8" spans="1:35" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="2"/>
       <c r="B8" s="10"/>
       <c r="C8" s="47" t="s">
@@ -40565,7 +40562,7 @@
       <c r="F8" s="17">
         <v>1</v>
       </c>
-      <c r="G8" s="68"/>
+      <c r="G8" s="64"/>
       <c r="I8" s="10"/>
       <c r="J8" s="47" t="s">
         <v>47</v>
@@ -40577,7 +40574,7 @@
       <c r="M8" s="17">
         <v>1</v>
       </c>
-      <c r="N8" s="68"/>
+      <c r="N8" s="64"/>
       <c r="P8" s="10"/>
       <c r="Q8" s="47" t="s">
         <v>47</v>
@@ -40589,7 +40586,7 @@
       <c r="T8" s="17">
         <v>1</v>
       </c>
-      <c r="U8" s="68"/>
+      <c r="U8" s="64"/>
       <c r="W8" s="10"/>
       <c r="X8" s="47" t="s">
         <v>47</v>
@@ -40601,7 +40598,7 @@
       <c r="AA8" s="17">
         <v>1</v>
       </c>
-      <c r="AB8" s="68"/>
+      <c r="AB8" s="64"/>
       <c r="AD8" s="10"/>
       <c r="AE8" s="47" t="s">
         <v>47</v>
@@ -40613,9 +40610,9 @@
       <c r="AH8" s="17">
         <v>1</v>
       </c>
-      <c r="AI8" s="68"/>
+      <c r="AI8" s="64"/>
     </row>
-    <row r="9" spans="1:35" ht="19.05" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
+    <row r="9" spans="1:35" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="2"/>
       <c r="B9" s="10"/>
       <c r="C9" s="18">
@@ -40624,11 +40621,13 @@
       <c r="D9" s="19">
         <v>0</v>
       </c>
-      <c r="E9" s="69" t="s">
+      <c r="E9" s="65" t="s">
         <v>43</v>
       </c>
-      <c r="F9" s="13"/>
-      <c r="G9" s="70" t="s">
+      <c r="F9" s="13">
+        <v>12</v>
+      </c>
+      <c r="G9" s="66" t="s">
         <v>49</v>
       </c>
       <c r="I9" s="10"/>
@@ -40638,11 +40637,13 @@
       <c r="K9" s="19">
         <v>2</v>
       </c>
-      <c r="L9" s="69" t="s">
+      <c r="L9" s="65" t="s">
         <v>43</v>
       </c>
-      <c r="M9" s="13"/>
-      <c r="N9" s="70" t="s">
+      <c r="M9" s="13">
+        <v>14</v>
+      </c>
+      <c r="N9" s="66" t="s">
         <v>49</v>
       </c>
       <c r="P9" s="10"/>
@@ -40652,11 +40653,13 @@
       <c r="R9" s="19">
         <v>-1</v>
       </c>
-      <c r="S9" s="69" t="s">
+      <c r="S9" s="65" t="s">
         <v>43</v>
       </c>
-      <c r="T9" s="13"/>
-      <c r="U9" s="70" t="s">
+      <c r="T9" s="13">
+        <v>11</v>
+      </c>
+      <c r="U9" s="66" t="s">
         <v>49</v>
       </c>
       <c r="W9" s="10"/>
@@ -40666,14 +40669,14 @@
       <c r="Y9" s="21">
         <v>2</v>
       </c>
-      <c r="Z9" s="69" t="s">
+      <c r="Z9" s="65" t="s">
         <v>43</v>
       </c>
       <c r="AA9" s="24">
         <f>X9*AA7+Y9</f>
         <v>14</v>
       </c>
-      <c r="AB9" s="71" t="s">
+      <c r="AB9" s="67" t="s">
         <v>52</v>
       </c>
       <c r="AD9" s="10"/>
@@ -40683,37 +40686,37 @@
       <c r="AF9" s="21">
         <v>2</v>
       </c>
-      <c r="AG9" s="69" t="s">
+      <c r="AG9" s="65" t="s">
         <v>43</v>
       </c>
       <c r="AH9" s="24">
         <f>AE9*AH7+AF9</f>
         <v>8</v>
       </c>
-      <c r="AI9" s="71" t="s">
+      <c r="AI9" s="67" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="10" spans="1:35" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
+    <row r="10" spans="1:35" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="2"/>
       <c r="B10" s="10"/>
       <c r="C10" s="1"/>
       <c r="D10" s="1"/>
       <c r="E10" s="1"/>
       <c r="F10" s="1"/>
-      <c r="G10" s="68"/>
+      <c r="G10" s="64"/>
       <c r="I10" s="10"/>
       <c r="J10" s="1"/>
       <c r="K10" s="1"/>
       <c r="L10" s="1"/>
       <c r="M10" s="1"/>
-      <c r="N10" s="68"/>
+      <c r="N10" s="64"/>
       <c r="P10" s="10"/>
       <c r="Q10" s="1"/>
       <c r="R10" s="1"/>
       <c r="S10" s="1"/>
       <c r="T10" s="1"/>
-      <c r="U10" s="68"/>
+      <c r="U10" s="64"/>
       <c r="W10" s="10"/>
       <c r="X10" s="22">
         <v>3</v>
@@ -40721,11 +40724,13 @@
       <c r="Y10" s="23">
         <v>-2</v>
       </c>
-      <c r="Z10" s="69" t="s">
+      <c r="Z10" s="65" t="s">
         <v>43</v>
       </c>
-      <c r="AA10" s="13"/>
-      <c r="AB10" s="70" t="s">
+      <c r="AA10" s="13">
+        <v>10</v>
+      </c>
+      <c r="AB10" s="66" t="s">
         <v>53</v>
       </c>
       <c r="AD10" s="10"/>
@@ -40735,302 +40740,304 @@
       <c r="AF10" s="26">
         <v>-2</v>
       </c>
-      <c r="AG10" s="69" t="s">
+      <c r="AG10" s="65" t="s">
         <v>43</v>
       </c>
       <c r="AH10" s="24">
         <f>AE10*AH7+AF10</f>
         <v>4</v>
       </c>
-      <c r="AI10" s="70" t="s">
+      <c r="AI10" s="66" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="11" spans="1:35" ht="19.05" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
+    <row r="11" spans="1:35" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="2"/>
-      <c r="B11" s="72" t="s">
+      <c r="B11" s="83" t="s">
         <v>45</v>
       </c>
-      <c r="C11" s="73"/>
-      <c r="D11" s="73"/>
-      <c r="E11" s="73"/>
-      <c r="F11" s="73"/>
-      <c r="G11" s="74"/>
-      <c r="I11" s="72" t="s">
+      <c r="C11" s="84"/>
+      <c r="D11" s="84"/>
+      <c r="E11" s="84"/>
+      <c r="F11" s="84"/>
+      <c r="G11" s="85"/>
+      <c r="I11" s="83" t="s">
         <v>45</v>
       </c>
-      <c r="J11" s="73"/>
-      <c r="K11" s="73"/>
-      <c r="L11" s="73"/>
-      <c r="M11" s="73"/>
-      <c r="N11" s="74"/>
-      <c r="P11" s="72" t="s">
+      <c r="J11" s="84"/>
+      <c r="K11" s="84"/>
+      <c r="L11" s="84"/>
+      <c r="M11" s="84"/>
+      <c r="N11" s="85"/>
+      <c r="P11" s="83" t="s">
         <v>45</v>
       </c>
-      <c r="Q11" s="73"/>
-      <c r="R11" s="73"/>
-      <c r="S11" s="73"/>
-      <c r="T11" s="73"/>
-      <c r="U11" s="74"/>
-      <c r="W11" s="75"/>
+      <c r="Q11" s="84"/>
+      <c r="R11" s="84"/>
+      <c r="S11" s="84"/>
+      <c r="T11" s="84"/>
+      <c r="U11" s="85"/>
+      <c r="W11" s="68"/>
       <c r="X11" s="1"/>
-      <c r="Y11" s="69"/>
+      <c r="Y11" s="65"/>
       <c r="Z11" s="1"/>
       <c r="AA11" s="1"/>
-      <c r="AB11" s="67"/>
-      <c r="AD11" s="75"/>
+      <c r="AB11" s="63"/>
+      <c r="AD11" s="68"/>
       <c r="AE11" s="22">
         <v>3</v>
       </c>
       <c r="AF11" s="23">
         <v>-4</v>
       </c>
-      <c r="AG11" s="69" t="s">
+      <c r="AG11" s="65" t="s">
         <v>43</v>
       </c>
-      <c r="AH11" s="13"/>
-      <c r="AI11" s="70" t="s">
+      <c r="AH11" s="13">
+        <v>2</v>
+      </c>
+      <c r="AI11" s="66" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="12" spans="1:35" ht="19.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="12" spans="1:35" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2"/>
       <c r="B12" s="15"/>
       <c r="C12" s="1"/>
-      <c r="D12" s="69"/>
+      <c r="D12" s="65"/>
       <c r="E12" s="1"/>
       <c r="F12" s="1"/>
-      <c r="G12" s="67"/>
+      <c r="G12" s="63"/>
       <c r="I12" s="15"/>
       <c r="J12" s="1"/>
-      <c r="K12" s="69"/>
+      <c r="K12" s="65"/>
       <c r="L12" s="1"/>
       <c r="M12" s="1"/>
-      <c r="N12" s="67"/>
+      <c r="N12" s="63"/>
       <c r="P12" s="15"/>
       <c r="Q12" s="1"/>
-      <c r="R12" s="69"/>
+      <c r="R12" s="65"/>
       <c r="S12" s="1"/>
       <c r="T12" s="1"/>
-      <c r="U12" s="67"/>
-      <c r="W12" s="76"/>
+      <c r="U12" s="63"/>
+      <c r="W12" s="69"/>
       <c r="X12" s="1"/>
-      <c r="Y12" s="69"/>
+      <c r="Y12" s="65"/>
       <c r="Z12" s="1"/>
       <c r="AA12" s="1"/>
-      <c r="AB12" s="77"/>
-      <c r="AD12" s="76"/>
+      <c r="AB12" s="70"/>
+      <c r="AD12" s="69"/>
       <c r="AE12" s="1"/>
-      <c r="AF12" s="69"/>
+      <c r="AF12" s="65"/>
       <c r="AG12" s="1"/>
       <c r="AH12" s="1"/>
-      <c r="AI12" s="77"/>
+      <c r="AI12" s="70"/>
     </row>
-    <row r="13" spans="1:35" ht="18" x14ac:dyDescent="0.55000000000000004">
+    <row r="13" spans="1:35" ht="19" x14ac:dyDescent="0.25">
       <c r="A13" s="2"/>
       <c r="B13" s="15"/>
       <c r="C13" s="1"/>
-      <c r="D13" s="69"/>
+      <c r="D13" s="65"/>
       <c r="E13" s="1"/>
       <c r="F13" s="1"/>
-      <c r="G13" s="67"/>
+      <c r="G13" s="63"/>
       <c r="I13" s="15"/>
       <c r="J13" s="1"/>
-      <c r="K13" s="69"/>
+      <c r="K13" s="65"/>
       <c r="L13" s="1"/>
       <c r="M13" s="1"/>
-      <c r="N13" s="67"/>
+      <c r="N13" s="63"/>
       <c r="P13" s="15"/>
       <c r="Q13" s="1"/>
-      <c r="R13" s="69"/>
+      <c r="R13" s="65"/>
       <c r="S13" s="1"/>
       <c r="T13" s="1"/>
-      <c r="U13" s="67"/>
+      <c r="U13" s="63"/>
       <c r="W13" s="15"/>
       <c r="X13" s="1"/>
-      <c r="Y13" s="69"/>
+      <c r="Y13" s="65"/>
       <c r="Z13" s="1"/>
       <c r="AA13" s="1"/>
-      <c r="AB13" s="67"/>
+      <c r="AB13" s="63"/>
       <c r="AD13" s="15"/>
       <c r="AE13" s="1"/>
-      <c r="AF13" s="69"/>
+      <c r="AF13" s="65"/>
       <c r="AG13" s="1"/>
       <c r="AH13" s="1"/>
-      <c r="AI13" s="67"/>
+      <c r="AI13" s="63"/>
     </row>
-    <row r="14" spans="1:35" ht="18" x14ac:dyDescent="0.55000000000000004">
+    <row r="14" spans="1:35" ht="19" x14ac:dyDescent="0.25">
       <c r="A14" s="2"/>
       <c r="B14" s="15"/>
       <c r="C14" s="1"/>
-      <c r="D14" s="69"/>
+      <c r="D14" s="65"/>
       <c r="E14" s="1"/>
       <c r="F14" s="1"/>
-      <c r="G14" s="67"/>
+      <c r="G14" s="63"/>
       <c r="I14" s="15"/>
       <c r="J14" s="1"/>
-      <c r="K14" s="69"/>
+      <c r="K14" s="65"/>
       <c r="L14" s="1"/>
       <c r="M14" s="1"/>
-      <c r="N14" s="67"/>
+      <c r="N14" s="63"/>
       <c r="P14" s="15"/>
       <c r="Q14" s="1"/>
-      <c r="R14" s="69"/>
+      <c r="R14" s="65"/>
       <c r="S14" s="1"/>
       <c r="T14" s="1"/>
-      <c r="U14" s="67"/>
+      <c r="U14" s="63"/>
       <c r="W14" s="15"/>
       <c r="X14" s="1"/>
-      <c r="Y14" s="69"/>
+      <c r="Y14" s="65"/>
       <c r="Z14" s="1"/>
       <c r="AA14" s="1"/>
-      <c r="AB14" s="67"/>
+      <c r="AB14" s="63"/>
       <c r="AD14" s="15"/>
       <c r="AE14" s="1"/>
-      <c r="AF14" s="69"/>
+      <c r="AF14" s="65"/>
       <c r="AG14" s="1"/>
       <c r="AH14" s="1"/>
-      <c r="AI14" s="67"/>
+      <c r="AI14" s="63"/>
     </row>
-    <row r="15" spans="1:35" ht="18" x14ac:dyDescent="0.55000000000000004">
+    <row r="15" spans="1:35" ht="19" x14ac:dyDescent="0.25">
       <c r="A15" s="2"/>
       <c r="B15" s="15"/>
       <c r="C15" s="1"/>
-      <c r="D15" s="69"/>
+      <c r="D15" s="65"/>
       <c r="E15" s="1"/>
       <c r="F15" s="1"/>
-      <c r="G15" s="67"/>
+      <c r="G15" s="63"/>
       <c r="I15" s="15"/>
       <c r="J15" s="1"/>
-      <c r="K15" s="69"/>
+      <c r="K15" s="65"/>
       <c r="L15" s="1"/>
       <c r="M15" s="1"/>
-      <c r="N15" s="67"/>
+      <c r="N15" s="63"/>
       <c r="P15" s="15"/>
       <c r="Q15" s="1"/>
-      <c r="R15" s="69"/>
+      <c r="R15" s="65"/>
       <c r="S15" s="1"/>
       <c r="T15" s="1"/>
-      <c r="U15" s="67"/>
+      <c r="U15" s="63"/>
       <c r="W15" s="15"/>
       <c r="X15" s="1"/>
-      <c r="Y15" s="69"/>
+      <c r="Y15" s="65"/>
       <c r="Z15" s="1"/>
       <c r="AA15" s="1"/>
-      <c r="AB15" s="67"/>
+      <c r="AB15" s="63"/>
       <c r="AD15" s="15"/>
       <c r="AE15" s="1"/>
-      <c r="AF15" s="69"/>
+      <c r="AF15" s="65"/>
       <c r="AG15" s="1"/>
       <c r="AH15" s="1"/>
-      <c r="AI15" s="67"/>
+      <c r="AI15" s="63"/>
     </row>
-    <row r="16" spans="1:35" ht="18" x14ac:dyDescent="0.55000000000000004">
+    <row r="16" spans="1:35" ht="19" x14ac:dyDescent="0.25">
       <c r="A16" s="2"/>
       <c r="B16" s="15"/>
       <c r="C16" s="1"/>
-      <c r="D16" s="69"/>
+      <c r="D16" s="65"/>
       <c r="E16" s="1"/>
       <c r="F16" s="1"/>
-      <c r="G16" s="67"/>
+      <c r="G16" s="63"/>
       <c r="I16" s="15"/>
       <c r="J16" s="1"/>
-      <c r="K16" s="69"/>
+      <c r="K16" s="65"/>
       <c r="L16" s="1"/>
       <c r="M16" s="1"/>
-      <c r="N16" s="67"/>
+      <c r="N16" s="63"/>
       <c r="P16" s="15"/>
       <c r="Q16" s="1"/>
-      <c r="R16" s="69"/>
+      <c r="R16" s="65"/>
       <c r="S16" s="1"/>
       <c r="T16" s="1"/>
-      <c r="U16" s="67"/>
+      <c r="U16" s="63"/>
       <c r="W16" s="15"/>
-      <c r="AB16" s="67"/>
+      <c r="AB16" s="63"/>
       <c r="AD16" s="15"/>
       <c r="AE16" s="1"/>
-      <c r="AF16" s="69"/>
+      <c r="AF16" s="65"/>
       <c r="AG16" s="1"/>
       <c r="AH16" s="1"/>
-      <c r="AI16" s="67"/>
+      <c r="AI16" s="63"/>
     </row>
-    <row r="17" spans="1:35" ht="18" x14ac:dyDescent="0.55000000000000004">
+    <row r="17" spans="1:35" ht="19" x14ac:dyDescent="0.25">
       <c r="A17" s="2"/>
       <c r="B17" s="15"/>
       <c r="C17" s="1"/>
-      <c r="D17" s="69"/>
+      <c r="D17" s="65"/>
       <c r="E17" s="1"/>
       <c r="F17" s="1"/>
-      <c r="G17" s="67"/>
+      <c r="G17" s="63"/>
       <c r="I17" s="15"/>
       <c r="J17" s="1"/>
-      <c r="K17" s="69"/>
+      <c r="K17" s="65"/>
       <c r="L17" s="1"/>
       <c r="M17" s="1"/>
-      <c r="N17" s="67"/>
+      <c r="N17" s="63"/>
       <c r="P17" s="15"/>
       <c r="Q17" s="1"/>
-      <c r="R17" s="69"/>
+      <c r="R17" s="65"/>
       <c r="S17" s="1"/>
       <c r="T17" s="1"/>
-      <c r="U17" s="67"/>
+      <c r="U17" s="63"/>
       <c r="W17" s="15"/>
       <c r="X17" s="2"/>
       <c r="Y17" s="2"/>
       <c r="Z17" s="2"/>
       <c r="AA17" s="2"/>
-      <c r="AB17" s="67"/>
+      <c r="AB17" s="63"/>
       <c r="AD17" s="15"/>
-      <c r="AI17" s="67"/>
+      <c r="AI17" s="63"/>
     </row>
-    <row r="18" spans="1:35" ht="18.399999999999999" thickBot="1" x14ac:dyDescent="0.6">
+    <row r="18" spans="1:35" ht="20" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="2"/>
       <c r="B18" s="11"/>
       <c r="C18" s="12"/>
       <c r="D18" s="12"/>
       <c r="E18" s="12"/>
       <c r="F18" s="12"/>
-      <c r="G18" s="78"/>
+      <c r="G18" s="71"/>
       <c r="I18" s="11"/>
       <c r="J18" s="12"/>
       <c r="K18" s="12"/>
       <c r="L18" s="12"/>
       <c r="M18" s="12"/>
-      <c r="N18" s="78"/>
+      <c r="N18" s="71"/>
       <c r="P18" s="11"/>
       <c r="Q18" s="12"/>
       <c r="R18" s="12"/>
       <c r="S18" s="12"/>
       <c r="T18" s="12"/>
-      <c r="U18" s="78"/>
+      <c r="U18" s="71"/>
       <c r="W18" s="11"/>
-      <c r="X18" s="79"/>
-      <c r="Y18" s="79"/>
-      <c r="Z18" s="79"/>
-      <c r="AA18" s="79"/>
-      <c r="AB18" s="78"/>
+      <c r="X18" s="72"/>
+      <c r="Y18" s="72"/>
+      <c r="Z18" s="72"/>
+      <c r="AA18" s="72"/>
+      <c r="AB18" s="71"/>
       <c r="AD18" s="10"/>
       <c r="AE18" s="2"/>
       <c r="AF18" s="2"/>
       <c r="AG18" s="2"/>
       <c r="AH18" s="2"/>
-      <c r="AI18" s="67"/>
+      <c r="AI18" s="63"/>
     </row>
-    <row r="19" spans="1:35" ht="18.399999999999999" thickBot="1" x14ac:dyDescent="0.6">
+    <row r="19" spans="1:35" ht="20" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="2"/>
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
       <c r="D19" s="2"/>
       <c r="E19" s="2"/>
       <c r="F19" s="2"/>
-      <c r="AD19" s="80"/>
-      <c r="AE19" s="79"/>
-      <c r="AF19" s="79"/>
-      <c r="AG19" s="79"/>
-      <c r="AH19" s="79"/>
-      <c r="AI19" s="78"/>
+      <c r="AD19" s="73"/>
+      <c r="AE19" s="72"/>
+      <c r="AF19" s="72"/>
+      <c r="AG19" s="72"/>
+      <c r="AH19" s="72"/>
+      <c r="AI19" s="71"/>
     </row>
-    <row r="20" spans="1:35" ht="18" x14ac:dyDescent="0.55000000000000004">
+    <row r="20" spans="1:35" ht="19" x14ac:dyDescent="0.25">
       <c r="A20" s="2"/>
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>
@@ -41060,43 +41067,41 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{028551B1-A2F3-B541-AC24-4DB708B5D11A}">
   <dimension ref="A1:AN21"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.5"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="11" style="63"/>
-    <col min="2" max="2" width="4.6875" style="63" customWidth="1"/>
-    <col min="3" max="5" width="4.5" style="63" customWidth="1"/>
-    <col min="6" max="6" width="4.6875" style="63" customWidth="1"/>
-    <col min="7" max="8" width="4.8125" style="63" customWidth="1"/>
-    <col min="9" max="9" width="10" style="63" customWidth="1"/>
-    <col min="10" max="10" width="4.8125" style="63" customWidth="1"/>
-    <col min="11" max="11" width="5" style="63" customWidth="1"/>
-    <col min="12" max="12" width="4.5" style="63" customWidth="1"/>
-    <col min="13" max="14" width="5" style="63" customWidth="1"/>
-    <col min="15" max="15" width="4.8125" style="63" customWidth="1"/>
-    <col min="16" max="16" width="4.5" style="63" customWidth="1"/>
-    <col min="17" max="17" width="10.5" style="63" customWidth="1"/>
-    <col min="18" max="18" width="4.5" style="63" customWidth="1"/>
-    <col min="19" max="19" width="4.6875" style="63" customWidth="1"/>
-    <col min="20" max="20" width="4.5" style="63" customWidth="1"/>
-    <col min="21" max="22" width="4.6875" style="63" customWidth="1"/>
-    <col min="23" max="24" width="4.5" style="63" customWidth="1"/>
-    <col min="25" max="25" width="10.1875" style="63" customWidth="1"/>
-    <col min="26" max="26" width="4.6875" style="63" customWidth="1"/>
-    <col min="27" max="27" width="4.3125" style="63" customWidth="1"/>
-    <col min="28" max="28" width="4.6875" style="63" customWidth="1"/>
-    <col min="29" max="29" width="4.8125" style="63" customWidth="1"/>
-    <col min="30" max="31" width="4.5" style="63" customWidth="1"/>
-    <col min="32" max="32" width="4.3125" style="63" customWidth="1"/>
-    <col min="33" max="33" width="10.3125" style="63" customWidth="1"/>
-    <col min="34" max="34" width="5" style="63" customWidth="1"/>
-    <col min="35" max="36" width="4.6875" style="63" customWidth="1"/>
-    <col min="37" max="37" width="4.5" style="63" customWidth="1"/>
-    <col min="38" max="38" width="4.6875" style="63" customWidth="1"/>
-    <col min="39" max="40" width="4.8125" style="63" customWidth="1"/>
-    <col min="41" max="16384" width="11" style="63"/>
+    <col min="2" max="2" width="4.6640625" customWidth="1"/>
+    <col min="3" max="5" width="4.5" customWidth="1"/>
+    <col min="6" max="6" width="4.6640625" customWidth="1"/>
+    <col min="7" max="8" width="4.83203125" customWidth="1"/>
+    <col min="9" max="9" width="10" customWidth="1"/>
+    <col min="10" max="10" width="4.83203125" customWidth="1"/>
+    <col min="11" max="11" width="5" customWidth="1"/>
+    <col min="12" max="12" width="4.5" customWidth="1"/>
+    <col min="13" max="14" width="5" customWidth="1"/>
+    <col min="15" max="15" width="4.83203125" customWidth="1"/>
+    <col min="16" max="16" width="4.5" customWidth="1"/>
+    <col min="17" max="17" width="10.5" customWidth="1"/>
+    <col min="18" max="18" width="4.5" customWidth="1"/>
+    <col min="19" max="19" width="4.6640625" customWidth="1"/>
+    <col min="20" max="20" width="4.5" customWidth="1"/>
+    <col min="21" max="22" width="4.6640625" customWidth="1"/>
+    <col min="23" max="24" width="4.5" customWidth="1"/>
+    <col min="25" max="25" width="10.1640625" customWidth="1"/>
+    <col min="26" max="26" width="4.6640625" customWidth="1"/>
+    <col min="27" max="27" width="4.33203125" customWidth="1"/>
+    <col min="28" max="28" width="4.6640625" customWidth="1"/>
+    <col min="29" max="29" width="4.83203125" customWidth="1"/>
+    <col min="30" max="31" width="4.5" customWidth="1"/>
+    <col min="32" max="32" width="4.33203125" customWidth="1"/>
+    <col min="33" max="33" width="10.33203125" customWidth="1"/>
+    <col min="34" max="34" width="5" customWidth="1"/>
+    <col min="35" max="36" width="4.6640625" customWidth="1"/>
+    <col min="37" max="37" width="4.5" customWidth="1"/>
+    <col min="38" max="38" width="4.6640625" customWidth="1"/>
+    <col min="39" max="40" width="4.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:40" s="2" customFormat="1" ht="19.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:40" s="2" customFormat="1" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>44</v>
       </c>
@@ -41108,11 +41113,11 @@
       <c r="N1" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="P1" s="81" t="s">
+      <c r="P1" s="74" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="3" spans="1:40" ht="18.399999999999999" thickBot="1" x14ac:dyDescent="0.6">
+    <row r="3" spans="1:40" ht="20" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="2" t="str">
         <f>IF(ISBLANK(G9)=TRUE,"NOT DONE",IF(B5=G9,"CORRECT", "INCORRECT"))</f>
         <v>NOT DONE</v>
@@ -41159,54 +41164,54 @@
       <c r="AL3" s="2"/>
       <c r="AM3" s="2"/>
     </row>
-    <row r="4" spans="1:40" ht="18" x14ac:dyDescent="0.55000000000000004">
-      <c r="B4" s="64" t="s">
+    <row r="4" spans="1:40" ht="19" x14ac:dyDescent="0.25">
+      <c r="B4" s="80" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="65"/>
-      <c r="D4" s="65"/>
-      <c r="E4" s="65"/>
-      <c r="F4" s="65"/>
-      <c r="G4" s="65"/>
-      <c r="H4" s="66"/>
-      <c r="J4" s="64" t="s">
+      <c r="C4" s="81"/>
+      <c r="D4" s="81"/>
+      <c r="E4" s="81"/>
+      <c r="F4" s="81"/>
+      <c r="G4" s="81"/>
+      <c r="H4" s="82"/>
+      <c r="J4" s="80" t="s">
         <v>6</v>
       </c>
-      <c r="K4" s="65"/>
-      <c r="L4" s="65"/>
-      <c r="M4" s="65"/>
-      <c r="N4" s="65"/>
-      <c r="O4" s="65"/>
-      <c r="P4" s="66"/>
-      <c r="R4" s="64" t="s">
+      <c r="K4" s="81"/>
+      <c r="L4" s="81"/>
+      <c r="M4" s="81"/>
+      <c r="N4" s="81"/>
+      <c r="O4" s="81"/>
+      <c r="P4" s="82"/>
+      <c r="R4" s="80" t="s">
         <v>7</v>
       </c>
-      <c r="S4" s="65"/>
-      <c r="T4" s="65"/>
-      <c r="U4" s="65"/>
-      <c r="V4" s="65"/>
-      <c r="W4" s="65"/>
-      <c r="X4" s="66"/>
-      <c r="Z4" s="64" t="s">
+      <c r="S4" s="81"/>
+      <c r="T4" s="81"/>
+      <c r="U4" s="81"/>
+      <c r="V4" s="81"/>
+      <c r="W4" s="81"/>
+      <c r="X4" s="82"/>
+      <c r="Z4" s="80" t="s">
         <v>8</v>
       </c>
-      <c r="AA4" s="65"/>
-      <c r="AB4" s="65"/>
-      <c r="AC4" s="65"/>
-      <c r="AD4" s="65"/>
-      <c r="AE4" s="65"/>
-      <c r="AF4" s="66"/>
-      <c r="AH4" s="64" t="s">
+      <c r="AA4" s="81"/>
+      <c r="AB4" s="81"/>
+      <c r="AC4" s="81"/>
+      <c r="AD4" s="81"/>
+      <c r="AE4" s="81"/>
+      <c r="AF4" s="82"/>
+      <c r="AH4" s="80" t="s">
         <v>9</v>
       </c>
-      <c r="AI4" s="65"/>
-      <c r="AJ4" s="65"/>
-      <c r="AK4" s="65"/>
-      <c r="AL4" s="65"/>
-      <c r="AM4" s="65"/>
-      <c r="AN4" s="66"/>
+      <c r="AI4" s="81"/>
+      <c r="AJ4" s="81"/>
+      <c r="AK4" s="81"/>
+      <c r="AL4" s="81"/>
+      <c r="AM4" s="81"/>
+      <c r="AN4" s="82"/>
     </row>
-    <row r="5" spans="1:40" ht="18" x14ac:dyDescent="0.55000000000000004">
+    <row r="5" spans="1:40" ht="19" x14ac:dyDescent="0.25">
       <c r="B5" s="14">
         <f>G6*C9+G7*D9+E9</f>
         <v>1</v>
@@ -41216,7 +41221,7 @@
       <c r="E5" s="2"/>
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
-      <c r="H5" s="67"/>
+      <c r="H5" s="63"/>
       <c r="J5" s="14">
         <f>O6*K9+O7*L9+M9</f>
         <v>9</v>
@@ -41226,7 +41231,7 @@
       <c r="M5" s="2"/>
       <c r="N5" s="2"/>
       <c r="O5" s="2"/>
-      <c r="P5" s="67"/>
+      <c r="P5" s="63"/>
       <c r="R5" s="14">
         <f>S9*W6+T9*W7+U9</f>
         <v>1</v>
@@ -41236,7 +41241,7 @@
       <c r="U5" s="2"/>
       <c r="V5" s="2"/>
       <c r="W5" s="2"/>
-      <c r="X5" s="67"/>
+      <c r="X5" s="63"/>
       <c r="Z5" s="9">
         <f>AA10*AE6+AB10*AE7+AC10</f>
         <v>3</v>
@@ -41246,7 +41251,7 @@
       <c r="AC5" s="2"/>
       <c r="AD5" s="2"/>
       <c r="AE5" s="2"/>
-      <c r="AF5" s="67"/>
+      <c r="AF5" s="63"/>
       <c r="AH5" s="9">
         <f>AI10*AM6+AJ10*AM7+AK10</f>
         <v>2</v>
@@ -41256,9 +41261,9 @@
       <c r="AK5" s="2"/>
       <c r="AL5" s="2"/>
       <c r="AM5" s="2"/>
-      <c r="AN5" s="67"/>
+      <c r="AN5" s="63"/>
     </row>
-    <row r="6" spans="1:40" ht="20" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="6" spans="1:40" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="10"/>
       <c r="C6" s="2"/>
       <c r="D6" s="1"/>
@@ -41267,7 +41272,7 @@
       <c r="G6" s="29">
         <v>2</v>
       </c>
-      <c r="H6" s="70" t="s">
+      <c r="H6" s="66" t="s">
         <v>55</v>
       </c>
       <c r="J6" s="10"/>
@@ -41278,7 +41283,7 @@
       <c r="O6" s="29">
         <v>2</v>
       </c>
-      <c r="P6" s="70" t="s">
+      <c r="P6" s="66" t="s">
         <v>55</v>
       </c>
       <c r="R6" s="10"/>
@@ -41289,7 +41294,7 @@
       <c r="W6" s="29">
         <v>2</v>
       </c>
-      <c r="X6" s="70" t="s">
+      <c r="X6" s="66" t="s">
         <v>55</v>
       </c>
       <c r="Z6" s="10"/>
@@ -41300,7 +41305,7 @@
       <c r="AE6" s="29">
         <v>2</v>
       </c>
-      <c r="AF6" s="70" t="s">
+      <c r="AF6" s="66" t="s">
         <v>55</v>
       </c>
       <c r="AH6" s="10"/>
@@ -41311,11 +41316,11 @@
       <c r="AM6" s="29">
         <v>3</v>
       </c>
-      <c r="AN6" s="70" t="s">
+      <c r="AN6" s="66" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="7" spans="1:40" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="7" spans="1:40" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="10"/>
       <c r="C7" s="2"/>
       <c r="D7" s="1"/>
@@ -41324,7 +41329,7 @@
       <c r="G7" s="29">
         <v>1</v>
       </c>
-      <c r="H7" s="70" t="s">
+      <c r="H7" s="66" t="s">
         <v>56</v>
       </c>
       <c r="J7" s="10"/>
@@ -41335,7 +41340,7 @@
       <c r="O7" s="29">
         <v>3</v>
       </c>
-      <c r="P7" s="70" t="s">
+      <c r="P7" s="66" t="s">
         <v>56</v>
       </c>
       <c r="R7" s="10"/>
@@ -41346,7 +41351,7 @@
       <c r="W7" s="29">
         <v>-1</v>
       </c>
-      <c r="X7" s="70" t="s">
+      <c r="X7" s="66" t="s">
         <v>56</v>
       </c>
       <c r="Z7" s="10"/>
@@ -41357,7 +41362,7 @@
       <c r="AE7" s="29">
         <v>1</v>
       </c>
-      <c r="AF7" s="70" t="s">
+      <c r="AF7" s="66" t="s">
         <v>56</v>
       </c>
       <c r="AH7" s="10"/>
@@ -41368,16 +41373,16 @@
       <c r="AM7" s="29">
         <v>2</v>
       </c>
-      <c r="AN7" s="70" t="s">
+      <c r="AN7" s="66" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="8" spans="1:40" ht="20" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
+    <row r="8" spans="1:40" ht="20" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B8" s="10"/>
-      <c r="C8" s="82" t="s">
+      <c r="C8" s="86" t="s">
         <v>47</v>
       </c>
-      <c r="D8" s="82"/>
+      <c r="D8" s="86"/>
       <c r="E8" s="47" t="s">
         <v>48</v>
       </c>
@@ -41385,12 +41390,12 @@
       <c r="G8" s="17">
         <v>1</v>
       </c>
-      <c r="H8" s="68"/>
+      <c r="H8" s="64"/>
       <c r="J8" s="10"/>
-      <c r="K8" s="82" t="s">
+      <c r="K8" s="86" t="s">
         <v>47</v>
       </c>
-      <c r="L8" s="82"/>
+      <c r="L8" s="86"/>
       <c r="M8" s="47" t="s">
         <v>48</v>
       </c>
@@ -41398,12 +41403,12 @@
       <c r="O8" s="17">
         <v>1</v>
       </c>
-      <c r="P8" s="68"/>
+      <c r="P8" s="64"/>
       <c r="R8" s="10"/>
-      <c r="S8" s="82" t="s">
+      <c r="S8" s="86" t="s">
         <v>47</v>
       </c>
-      <c r="T8" s="82"/>
+      <c r="T8" s="86"/>
       <c r="U8" s="47" t="s">
         <v>48</v>
       </c>
@@ -41411,12 +41416,12 @@
       <c r="W8" s="17">
         <v>1</v>
       </c>
-      <c r="X8" s="68"/>
+      <c r="X8" s="64"/>
       <c r="Z8" s="10"/>
-      <c r="AA8" s="82" t="s">
+      <c r="AA8" s="86" t="s">
         <v>47</v>
       </c>
-      <c r="AB8" s="82"/>
+      <c r="AB8" s="86"/>
       <c r="AC8" s="47" t="s">
         <v>48</v>
       </c>
@@ -41424,12 +41429,12 @@
       <c r="AE8" s="17">
         <v>1</v>
       </c>
-      <c r="AF8" s="68"/>
+      <c r="AF8" s="64"/>
       <c r="AH8" s="10"/>
-      <c r="AI8" s="82" t="s">
+      <c r="AI8" s="86" t="s">
         <v>47</v>
       </c>
-      <c r="AJ8" s="82"/>
+      <c r="AJ8" s="86"/>
       <c r="AK8" s="47" t="s">
         <v>48</v>
       </c>
@@ -41437,9 +41442,9 @@
       <c r="AM8" s="17">
         <v>1</v>
       </c>
-      <c r="AN8" s="68"/>
+      <c r="AN8" s="64"/>
     </row>
-    <row r="9" spans="1:40" ht="21.4" thickBot="1" x14ac:dyDescent="0.6">
+    <row r="9" spans="1:40" ht="20" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B9" s="10"/>
       <c r="C9" s="30">
         <v>1</v>
@@ -41454,7 +41459,7 @@
         <v>43</v>
       </c>
       <c r="G9" s="13"/>
-      <c r="H9" s="70" t="s">
+      <c r="H9" s="66" t="s">
         <v>49</v>
       </c>
       <c r="J9" s="10"/>
@@ -41471,7 +41476,7 @@
         <v>43</v>
       </c>
       <c r="O9" s="13"/>
-      <c r="P9" s="70" t="s">
+      <c r="P9" s="66" t="s">
         <v>49</v>
       </c>
       <c r="R9" s="10"/>
@@ -41488,7 +41493,7 @@
         <v>43</v>
       </c>
       <c r="W9" s="13"/>
-      <c r="X9" s="71" t="s">
+      <c r="X9" s="67" t="s">
         <v>52</v>
       </c>
       <c r="Z9" s="10"/>
@@ -41508,7 +41513,7 @@
         <f>AA9*AE6+AB9*AE7+AC9</f>
         <v>5</v>
       </c>
-      <c r="AF9" s="71" t="s">
+      <c r="AF9" s="67" t="s">
         <v>52</v>
       </c>
       <c r="AH9" s="10"/>
@@ -41528,24 +41533,24 @@
         <f>AI9*AM6+AJ9*AM7+AK9</f>
         <v>5</v>
       </c>
-      <c r="AN9" s="71" t="s">
+      <c r="AN9" s="67" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="10" spans="1:40" ht="21.4" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="B10" s="75"/>
+    <row r="10" spans="1:40" ht="20" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B10" s="68"/>
       <c r="D10" s="1"/>
-      <c r="E10" s="69"/>
+      <c r="E10" s="65"/>
       <c r="F10" s="1"/>
       <c r="G10" s="1"/>
-      <c r="H10" s="67"/>
-      <c r="J10" s="75"/>
+      <c r="H10" s="63"/>
+      <c r="J10" s="68"/>
       <c r="L10" s="1"/>
-      <c r="M10" s="69"/>
+      <c r="M10" s="65"/>
       <c r="N10" s="1"/>
       <c r="O10" s="1"/>
-      <c r="P10" s="67"/>
-      <c r="R10" s="75"/>
+      <c r="P10" s="63"/>
+      <c r="R10" s="68"/>
       <c r="S10" s="22">
         <v>1</v>
       </c>
@@ -41562,10 +41567,10 @@
         <f>S10*W6+T10*W7+U10</f>
         <v>3</v>
       </c>
-      <c r="X10" s="71" t="s">
+      <c r="X10" s="67" t="s">
         <v>53</v>
       </c>
-      <c r="Z10" s="75"/>
+      <c r="Z10" s="68"/>
       <c r="AA10" s="34">
         <v>1</v>
       </c>
@@ -41579,10 +41584,10 @@
         <v>43</v>
       </c>
       <c r="AE10" s="56"/>
-      <c r="AF10" s="71" t="s">
+      <c r="AF10" s="67" t="s">
         <v>53</v>
       </c>
-      <c r="AH10" s="75"/>
+      <c r="AH10" s="68"/>
       <c r="AI10" s="25">
         <v>0</v>
       </c>
@@ -41596,30 +41601,30 @@
         <v>43</v>
       </c>
       <c r="AM10" s="13"/>
-      <c r="AN10" s="71" t="s">
+      <c r="AN10" s="67" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="11" spans="1:40" ht="21.4" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="B11" s="76"/>
-      <c r="C11" s="83"/>
+    <row r="11" spans="1:40" ht="20" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B11" s="69"/>
+      <c r="C11" s="75"/>
       <c r="D11" s="1"/>
-      <c r="E11" s="69"/>
+      <c r="E11" s="65"/>
       <c r="F11" s="1"/>
       <c r="G11" s="1"/>
-      <c r="H11" s="77"/>
-      <c r="J11" s="76"/>
-      <c r="K11" s="83"/>
+      <c r="H11" s="70"/>
+      <c r="J11" s="69"/>
+      <c r="K11" s="75"/>
       <c r="L11" s="1"/>
-      <c r="M11" s="69"/>
+      <c r="M11" s="65"/>
       <c r="N11" s="1"/>
       <c r="O11" s="1"/>
-      <c r="P11" s="77"/>
-      <c r="R11" s="76"/>
-      <c r="X11" s="77"/>
-      <c r="Z11" s="76"/>
-      <c r="AF11" s="77"/>
-      <c r="AH11" s="76"/>
+      <c r="P11" s="70"/>
+      <c r="R11" s="69"/>
+      <c r="X11" s="70"/>
+      <c r="Z11" s="69"/>
+      <c r="AF11" s="70"/>
+      <c r="AH11" s="69"/>
       <c r="AI11" s="34">
         <v>1</v>
       </c>
@@ -41636,250 +41641,250 @@
         <f>AI11*AM6+AM7*AJ11+AK11</f>
         <v>1</v>
       </c>
-      <c r="AN11" s="71" t="s">
+      <c r="AN11" s="67" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="12" spans="1:40" ht="18" x14ac:dyDescent="0.55000000000000004">
+    <row r="12" spans="1:40" ht="19" x14ac:dyDescent="0.25">
       <c r="B12" s="15"/>
       <c r="C12" s="1"/>
       <c r="D12" s="1"/>
-      <c r="E12" s="69"/>
+      <c r="E12" s="65"/>
       <c r="F12" s="1"/>
       <c r="G12" s="1"/>
-      <c r="H12" s="67"/>
+      <c r="H12" s="63"/>
       <c r="J12" s="15"/>
       <c r="K12" s="1"/>
       <c r="L12" s="1"/>
-      <c r="M12" s="69"/>
+      <c r="M12" s="65"/>
       <c r="N12" s="1"/>
       <c r="O12" s="1"/>
-      <c r="P12" s="67"/>
-      <c r="R12" s="75"/>
+      <c r="P12" s="63"/>
+      <c r="R12" s="68"/>
       <c r="S12" s="1"/>
-      <c r="T12" s="83"/>
+      <c r="T12" s="75"/>
       <c r="U12" s="1"/>
-      <c r="V12" s="69"/>
+      <c r="V12" s="65"/>
       <c r="W12" s="1"/>
       <c r="X12" s="39"/>
-      <c r="Z12" s="75"/>
+      <c r="Z12" s="68"/>
       <c r="AA12" s="1"/>
-      <c r="AB12" s="83"/>
+      <c r="AB12" s="75"/>
       <c r="AC12" s="1"/>
-      <c r="AD12" s="69"/>
+      <c r="AD12" s="65"/>
       <c r="AE12" s="1"/>
       <c r="AF12" s="39"/>
-      <c r="AH12" s="75"/>
-      <c r="AN12" s="67"/>
+      <c r="AH12" s="68"/>
+      <c r="AN12" s="63"/>
     </row>
-    <row r="13" spans="1:40" ht="18" x14ac:dyDescent="0.55000000000000004">
+    <row r="13" spans="1:40" ht="19" x14ac:dyDescent="0.25">
       <c r="B13" s="15"/>
       <c r="C13" s="1"/>
       <c r="D13" s="1"/>
-      <c r="E13" s="69"/>
+      <c r="E13" s="65"/>
       <c r="F13" s="1"/>
       <c r="G13" s="1"/>
-      <c r="H13" s="67"/>
+      <c r="H13" s="63"/>
       <c r="J13" s="15"/>
       <c r="K13" s="1"/>
       <c r="L13" s="1"/>
-      <c r="M13" s="69"/>
+      <c r="M13" s="65"/>
       <c r="N13" s="1"/>
       <c r="O13" s="1"/>
-      <c r="P13" s="67"/>
-      <c r="R13" s="75"/>
+      <c r="P13" s="63"/>
+      <c r="R13" s="68"/>
       <c r="S13" s="1"/>
       <c r="T13" s="1"/>
       <c r="U13" s="1"/>
-      <c r="V13" s="69"/>
+      <c r="V13" s="65"/>
       <c r="W13" s="1"/>
       <c r="X13" s="39"/>
-      <c r="Z13" s="75"/>
+      <c r="Z13" s="68"/>
       <c r="AA13" s="1"/>
       <c r="AB13" s="1"/>
       <c r="AC13" s="1"/>
-      <c r="AD13" s="69"/>
+      <c r="AD13" s="65"/>
       <c r="AE13" s="1"/>
       <c r="AF13" s="39"/>
-      <c r="AH13" s="75"/>
+      <c r="AH13" s="68"/>
       <c r="AN13" s="39"/>
     </row>
-    <row r="14" spans="1:40" ht="18" x14ac:dyDescent="0.55000000000000004">
+    <row r="14" spans="1:40" ht="19" x14ac:dyDescent="0.25">
       <c r="B14" s="15"/>
       <c r="C14" s="1"/>
       <c r="D14" s="1"/>
-      <c r="E14" s="69"/>
+      <c r="E14" s="65"/>
       <c r="F14" s="1"/>
       <c r="G14" s="1"/>
-      <c r="H14" s="67"/>
+      <c r="H14" s="63"/>
       <c r="J14" s="15"/>
       <c r="K14" s="1"/>
       <c r="L14" s="1"/>
-      <c r="M14" s="69"/>
+      <c r="M14" s="65"/>
       <c r="N14" s="1"/>
       <c r="O14" s="1"/>
-      <c r="P14" s="67"/>
-      <c r="R14" s="75"/>
+      <c r="P14" s="63"/>
+      <c r="R14" s="68"/>
       <c r="S14" s="1"/>
       <c r="T14" s="1"/>
       <c r="U14" s="1"/>
-      <c r="V14" s="69"/>
+      <c r="V14" s="65"/>
       <c r="W14" s="1"/>
       <c r="X14" s="39"/>
-      <c r="Z14" s="75"/>
+      <c r="Z14" s="68"/>
       <c r="AA14" s="1"/>
       <c r="AB14" s="1"/>
       <c r="AC14" s="1"/>
-      <c r="AD14" s="69"/>
+      <c r="AD14" s="65"/>
       <c r="AE14" s="1"/>
       <c r="AF14" s="39"/>
-      <c r="AH14" s="75"/>
+      <c r="AH14" s="68"/>
       <c r="AN14" s="39"/>
     </row>
-    <row r="15" spans="1:40" ht="18" x14ac:dyDescent="0.55000000000000004">
+    <row r="15" spans="1:40" ht="19" x14ac:dyDescent="0.25">
       <c r="B15" s="15"/>
       <c r="C15" s="1"/>
-      <c r="H15" s="67"/>
+      <c r="H15" s="63"/>
       <c r="J15" s="15"/>
       <c r="K15" s="1"/>
-      <c r="P15" s="67"/>
-      <c r="R15" s="75"/>
+      <c r="P15" s="63"/>
+      <c r="R15" s="68"/>
       <c r="S15" s="1"/>
       <c r="T15" s="1"/>
       <c r="U15" s="1"/>
-      <c r="V15" s="69"/>
+      <c r="V15" s="65"/>
       <c r="W15" s="1"/>
       <c r="X15" s="39"/>
-      <c r="Z15" s="75"/>
+      <c r="Z15" s="68"/>
       <c r="AA15" s="1"/>
       <c r="AB15" s="1"/>
       <c r="AC15" s="1"/>
-      <c r="AD15" s="69"/>
+      <c r="AD15" s="65"/>
       <c r="AE15" s="1"/>
       <c r="AF15" s="39"/>
-      <c r="AH15" s="75"/>
+      <c r="AH15" s="68"/>
       <c r="AN15" s="39"/>
     </row>
-    <row r="16" spans="1:40" ht="18" x14ac:dyDescent="0.55000000000000004">
+    <row r="16" spans="1:40" ht="19" x14ac:dyDescent="0.25">
       <c r="B16" s="15"/>
       <c r="C16" s="1"/>
-      <c r="H16" s="67"/>
+      <c r="H16" s="63"/>
       <c r="J16" s="15"/>
       <c r="K16" s="1"/>
-      <c r="P16" s="67"/>
-      <c r="R16" s="75"/>
+      <c r="P16" s="63"/>
+      <c r="R16" s="68"/>
       <c r="S16" s="1"/>
       <c r="T16" s="1"/>
-      <c r="X16" s="67"/>
-      <c r="Z16" s="75"/>
+      <c r="X16" s="63"/>
+      <c r="Z16" s="68"/>
       <c r="AA16" s="1"/>
       <c r="AB16" s="1"/>
-      <c r="AF16" s="67"/>
-      <c r="AH16" s="75"/>
+      <c r="AF16" s="63"/>
+      <c r="AH16" s="68"/>
       <c r="AN16" s="39"/>
     </row>
-    <row r="17" spans="2:40" ht="18" x14ac:dyDescent="0.55000000000000004">
+    <row r="17" spans="2:40" ht="19" x14ac:dyDescent="0.25">
       <c r="B17" s="15"/>
       <c r="C17" s="1"/>
-      <c r="H17" s="67"/>
+      <c r="H17" s="63"/>
       <c r="J17" s="15"/>
       <c r="K17" s="1"/>
-      <c r="P17" s="67"/>
-      <c r="R17" s="75"/>
+      <c r="P17" s="63"/>
+      <c r="R17" s="68"/>
       <c r="S17" s="1"/>
       <c r="T17" s="1"/>
-      <c r="X17" s="67"/>
-      <c r="Z17" s="75"/>
+      <c r="X17" s="63"/>
+      <c r="Z17" s="68"/>
       <c r="AA17" s="1"/>
       <c r="AB17" s="1"/>
-      <c r="AF17" s="67"/>
-      <c r="AH17" s="75"/>
-      <c r="AN17" s="67"/>
+      <c r="AF17" s="63"/>
+      <c r="AH17" s="68"/>
+      <c r="AN17" s="63"/>
     </row>
-    <row r="18" spans="2:40" ht="18" x14ac:dyDescent="0.55000000000000004">
+    <row r="18" spans="2:40" ht="19" x14ac:dyDescent="0.25">
       <c r="B18" s="15"/>
       <c r="C18" s="1"/>
       <c r="D18" s="2"/>
       <c r="E18" s="2"/>
       <c r="F18" s="2"/>
       <c r="G18" s="2"/>
-      <c r="H18" s="67"/>
+      <c r="H18" s="63"/>
       <c r="J18" s="15"/>
       <c r="K18" s="1"/>
       <c r="L18" s="2"/>
       <c r="M18" s="2"/>
       <c r="N18" s="2"/>
       <c r="O18" s="2"/>
-      <c r="P18" s="67"/>
-      <c r="R18" s="75"/>
+      <c r="P18" s="63"/>
+      <c r="R18" s="68"/>
       <c r="S18" s="1"/>
       <c r="T18" s="1"/>
-      <c r="X18" s="67"/>
-      <c r="Z18" s="75"/>
+      <c r="X18" s="63"/>
+      <c r="Z18" s="68"/>
       <c r="AA18" s="1"/>
       <c r="AB18" s="1"/>
-      <c r="AF18" s="67"/>
-      <c r="AH18" s="75"/>
-      <c r="AN18" s="67"/>
+      <c r="AF18" s="63"/>
+      <c r="AH18" s="68"/>
+      <c r="AN18" s="63"/>
     </row>
-    <row r="19" spans="2:40" ht="18.399999999999999" thickBot="1" x14ac:dyDescent="0.6">
+    <row r="19" spans="2:40" ht="20" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B19" s="11"/>
       <c r="C19" s="12"/>
-      <c r="D19" s="79"/>
-      <c r="E19" s="79"/>
-      <c r="F19" s="79"/>
-      <c r="G19" s="79"/>
-      <c r="H19" s="78"/>
+      <c r="D19" s="72"/>
+      <c r="E19" s="72"/>
+      <c r="F19" s="72"/>
+      <c r="G19" s="72"/>
+      <c r="H19" s="71"/>
       <c r="J19" s="11"/>
       <c r="K19" s="12"/>
-      <c r="L19" s="79"/>
-      <c r="M19" s="79"/>
-      <c r="N19" s="79"/>
-      <c r="O19" s="79"/>
-      <c r="P19" s="78"/>
-      <c r="R19" s="75"/>
+      <c r="L19" s="72"/>
+      <c r="M19" s="72"/>
+      <c r="N19" s="72"/>
+      <c r="O19" s="72"/>
+      <c r="P19" s="71"/>
+      <c r="R19" s="68"/>
       <c r="S19" s="2"/>
       <c r="T19" s="1"/>
       <c r="U19" s="2"/>
       <c r="V19" s="2"/>
       <c r="W19" s="2"/>
       <c r="X19" s="40"/>
-      <c r="Z19" s="75"/>
+      <c r="Z19" s="68"/>
       <c r="AA19" s="2"/>
       <c r="AB19" s="1"/>
       <c r="AC19" s="2"/>
       <c r="AD19" s="2"/>
       <c r="AE19" s="2"/>
       <c r="AF19" s="40"/>
-      <c r="AH19" s="75"/>
-      <c r="AN19" s="67"/>
+      <c r="AH19" s="68"/>
+      <c r="AN19" s="63"/>
     </row>
-    <row r="20" spans="2:40" ht="18.399999999999999" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="R20" s="80"/>
-      <c r="S20" s="79"/>
+    <row r="20" spans="2:40" ht="20" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R20" s="73"/>
+      <c r="S20" s="72"/>
       <c r="T20" s="12"/>
-      <c r="U20" s="79"/>
-      <c r="V20" s="79"/>
-      <c r="W20" s="79"/>
-      <c r="X20" s="78"/>
-      <c r="Z20" s="80"/>
-      <c r="AA20" s="79"/>
+      <c r="U20" s="72"/>
+      <c r="V20" s="72"/>
+      <c r="W20" s="72"/>
+      <c r="X20" s="71"/>
+      <c r="Z20" s="73"/>
+      <c r="AA20" s="72"/>
       <c r="AB20" s="12"/>
-      <c r="AC20" s="79"/>
-      <c r="AD20" s="79"/>
-      <c r="AE20" s="79"/>
-      <c r="AF20" s="78"/>
-      <c r="AH20" s="75"/>
+      <c r="AC20" s="72"/>
+      <c r="AD20" s="72"/>
+      <c r="AE20" s="72"/>
+      <c r="AF20" s="71"/>
+      <c r="AH20" s="68"/>
       <c r="AN20" s="40"/>
     </row>
-    <row r="21" spans="2:40" ht="16.149999999999999" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="AH21" s="80"/>
-      <c r="AI21" s="79"/>
-      <c r="AJ21" s="79"/>
-      <c r="AK21" s="79"/>
-      <c r="AL21" s="79"/>
-      <c r="AM21" s="79"/>
-      <c r="AN21" s="78"/>
+    <row r="21" spans="2:40" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="AH21" s="73"/>
+      <c r="AI21" s="72"/>
+      <c r="AJ21" s="72"/>
+      <c r="AK21" s="72"/>
+      <c r="AL21" s="72"/>
+      <c r="AM21" s="72"/>
+      <c r="AN21" s="71"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -41905,42 +41910,38 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{48F5CA51-81E0-194E-83C9-2EB882D0E921}">
   <dimension ref="A1:AQ21"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.5"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="11" style="63"/>
-    <col min="2" max="2" width="4.8125" style="63" customWidth="1"/>
-    <col min="3" max="3" width="4.6875" style="63" customWidth="1"/>
-    <col min="4" max="4" width="4.5" style="63" customWidth="1"/>
-    <col min="5" max="5" width="4.3125" style="63" customWidth="1"/>
-    <col min="6" max="6" width="4.6875" style="63" customWidth="1"/>
-    <col min="7" max="7" width="4.5" style="63" customWidth="1"/>
-    <col min="8" max="8" width="4.6875" style="63" customWidth="1"/>
-    <col min="9" max="9" width="9.6875" style="63" customWidth="1"/>
-    <col min="10" max="11" width="4.5" style="63" customWidth="1"/>
-    <col min="12" max="13" width="4.6875" style="63" customWidth="1"/>
-    <col min="14" max="14" width="4" style="63" customWidth="1"/>
-    <col min="15" max="15" width="4.3125" style="63" customWidth="1"/>
-    <col min="16" max="17" width="4.5" style="63" customWidth="1"/>
-    <col min="18" max="18" width="9.8125" style="63" customWidth="1"/>
-    <col min="19" max="22" width="4.6875" style="63" customWidth="1"/>
-    <col min="23" max="23" width="4.3125" style="63" customWidth="1"/>
-    <col min="24" max="24" width="4.6875" style="63" customWidth="1"/>
-    <col min="25" max="25" width="4.3125" style="63" customWidth="1"/>
-    <col min="26" max="26" width="4.6875" style="63" customWidth="1"/>
-    <col min="27" max="27" width="11" style="63"/>
-    <col min="28" max="32" width="4.6875" style="63" customWidth="1"/>
-    <col min="33" max="35" width="4.5" style="63" customWidth="1"/>
-    <col min="36" max="36" width="11" style="63"/>
-    <col min="37" max="37" width="5.1875" style="63" customWidth="1"/>
-    <col min="38" max="38" width="5" style="63" customWidth="1"/>
-    <col min="39" max="39" width="4.8125" style="63" customWidth="1"/>
-    <col min="40" max="40" width="5" style="63" customWidth="1"/>
-    <col min="41" max="42" width="4.8125" style="63" customWidth="1"/>
-    <col min="43" max="43" width="5" style="63" customWidth="1"/>
-    <col min="44" max="16384" width="11" style="63"/>
+    <col min="2" max="2" width="4.83203125" customWidth="1"/>
+    <col min="3" max="3" width="4.6640625" customWidth="1"/>
+    <col min="4" max="4" width="4.5" customWidth="1"/>
+    <col min="5" max="5" width="4.33203125" customWidth="1"/>
+    <col min="6" max="6" width="4.6640625" customWidth="1"/>
+    <col min="7" max="7" width="4.5" customWidth="1"/>
+    <col min="8" max="8" width="4.6640625" customWidth="1"/>
+    <col min="9" max="9" width="9.6640625" customWidth="1"/>
+    <col min="10" max="11" width="4.5" customWidth="1"/>
+    <col min="12" max="13" width="4.6640625" customWidth="1"/>
+    <col min="14" max="14" width="4" customWidth="1"/>
+    <col min="15" max="15" width="4.33203125" customWidth="1"/>
+    <col min="16" max="17" width="4.5" customWidth="1"/>
+    <col min="18" max="18" width="9.83203125" customWidth="1"/>
+    <col min="19" max="22" width="4.6640625" customWidth="1"/>
+    <col min="23" max="23" width="4.33203125" customWidth="1"/>
+    <col min="24" max="24" width="4.6640625" customWidth="1"/>
+    <col min="25" max="25" width="4.33203125" customWidth="1"/>
+    <col min="26" max="26" width="4.6640625" customWidth="1"/>
+    <col min="28" max="32" width="4.6640625" customWidth="1"/>
+    <col min="33" max="35" width="4.5" customWidth="1"/>
+    <col min="37" max="37" width="5.1640625" customWidth="1"/>
+    <col min="38" max="38" width="5" customWidth="1"/>
+    <col min="39" max="39" width="4.83203125" customWidth="1"/>
+    <col min="40" max="40" width="5" customWidth="1"/>
+    <col min="41" max="42" width="4.83203125" customWidth="1"/>
+    <col min="43" max="43" width="5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:43" s="2" customFormat="1" ht="19" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>51</v>
       </c>
@@ -41956,11 +41957,11 @@
       <c r="P1" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="S1" s="81" t="s">
+      <c r="S1" s="74" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="3" spans="1:43" ht="18.399999999999999" thickBot="1" x14ac:dyDescent="0.6">
+    <row r="3" spans="1:43" ht="20" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="2" t="str">
         <f>IF(ISBLANK(G11)=TRUE,"NOT DONE",IF(B5=G11,"CORRECT", "INCORRECT"))</f>
         <v>NOT DONE</v>
@@ -42012,57 +42013,57 @@
       <c r="AO3" s="2"/>
       <c r="AP3" s="2"/>
     </row>
-    <row r="4" spans="1:43" ht="18" x14ac:dyDescent="0.55000000000000004">
-      <c r="B4" s="64" t="s">
+    <row r="4" spans="1:43" ht="19" x14ac:dyDescent="0.25">
+      <c r="B4" s="80" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="65"/>
-      <c r="D4" s="65"/>
-      <c r="E4" s="65"/>
-      <c r="F4" s="65"/>
-      <c r="G4" s="65"/>
-      <c r="H4" s="66"/>
-      <c r="J4" s="64" t="s">
+      <c r="C4" s="81"/>
+      <c r="D4" s="81"/>
+      <c r="E4" s="81"/>
+      <c r="F4" s="81"/>
+      <c r="G4" s="81"/>
+      <c r="H4" s="82"/>
+      <c r="J4" s="80" t="s">
         <v>11</v>
       </c>
-      <c r="K4" s="65"/>
-      <c r="L4" s="65"/>
-      <c r="M4" s="65"/>
-      <c r="N4" s="65"/>
-      <c r="O4" s="65"/>
-      <c r="P4" s="65"/>
-      <c r="Q4" s="66"/>
-      <c r="S4" s="64" t="s">
+      <c r="K4" s="81"/>
+      <c r="L4" s="81"/>
+      <c r="M4" s="81"/>
+      <c r="N4" s="81"/>
+      <c r="O4" s="81"/>
+      <c r="P4" s="81"/>
+      <c r="Q4" s="82"/>
+      <c r="S4" s="80" t="s">
         <v>12</v>
       </c>
-      <c r="T4" s="65"/>
-      <c r="U4" s="65"/>
-      <c r="V4" s="65"/>
-      <c r="W4" s="65"/>
-      <c r="X4" s="65"/>
-      <c r="Y4" s="65"/>
-      <c r="Z4" s="66"/>
-      <c r="AB4" s="64" t="s">
+      <c r="T4" s="81"/>
+      <c r="U4" s="81"/>
+      <c r="V4" s="81"/>
+      <c r="W4" s="81"/>
+      <c r="X4" s="81"/>
+      <c r="Y4" s="81"/>
+      <c r="Z4" s="82"/>
+      <c r="AB4" s="80" t="s">
         <v>13</v>
       </c>
-      <c r="AC4" s="65"/>
-      <c r="AD4" s="65"/>
-      <c r="AE4" s="65"/>
-      <c r="AF4" s="65"/>
-      <c r="AG4" s="65"/>
-      <c r="AH4" s="65"/>
-      <c r="AI4" s="66"/>
-      <c r="AK4" s="64" t="s">
+      <c r="AC4" s="81"/>
+      <c r="AD4" s="81"/>
+      <c r="AE4" s="81"/>
+      <c r="AF4" s="81"/>
+      <c r="AG4" s="81"/>
+      <c r="AH4" s="81"/>
+      <c r="AI4" s="82"/>
+      <c r="AK4" s="80" t="s">
         <v>14</v>
       </c>
-      <c r="AL4" s="65"/>
-      <c r="AM4" s="65"/>
-      <c r="AN4" s="65"/>
-      <c r="AO4" s="65"/>
-      <c r="AP4" s="65"/>
-      <c r="AQ4" s="66"/>
+      <c r="AL4" s="81"/>
+      <c r="AM4" s="81"/>
+      <c r="AN4" s="81"/>
+      <c r="AO4" s="81"/>
+      <c r="AP4" s="81"/>
+      <c r="AQ4" s="82"/>
     </row>
-    <row r="5" spans="1:43" ht="18" x14ac:dyDescent="0.55000000000000004">
+    <row r="5" spans="1:43" ht="19" x14ac:dyDescent="0.25">
       <c r="B5" s="9">
         <f>C11*G6+D11*G7+E11</f>
         <v>3</v>
@@ -42072,7 +42073,7 @@
       <c r="E5" s="2"/>
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
-      <c r="H5" s="67"/>
+      <c r="H5" s="63"/>
       <c r="J5" s="9">
         <f>K10*P6+L10*P7+M10*P8+N10</f>
         <v>6</v>
@@ -42083,7 +42084,7 @@
       <c r="N5" s="2"/>
       <c r="O5" s="2"/>
       <c r="P5" s="2"/>
-      <c r="Q5" s="67"/>
+      <c r="Q5" s="63"/>
       <c r="S5" s="9">
         <f>T11*Y6+U11*Y7+V11*Y8+W11</f>
         <v>4</v>
@@ -42094,7 +42095,7 @@
       <c r="W5" s="2"/>
       <c r="X5" s="2"/>
       <c r="Y5" s="2"/>
-      <c r="Z5" s="67"/>
+      <c r="Z5" s="63"/>
       <c r="AB5" s="9">
         <f>AC11*AH6+AD11*AH7+AE11*AH8+AF11</f>
         <v>3</v>
@@ -42105,7 +42106,7 @@
       <c r="AF5" s="2"/>
       <c r="AG5" s="2"/>
       <c r="AH5" s="2"/>
-      <c r="AI5" s="67"/>
+      <c r="AI5" s="63"/>
       <c r="AK5" s="14">
         <f>(AP9-AN9-AP7*AM9)/AP6</f>
         <v>1</v>
@@ -42115,9 +42116,9 @@
       <c r="AN5" s="2"/>
       <c r="AO5" s="2"/>
       <c r="AP5" s="2"/>
-      <c r="AQ5" s="67"/>
+      <c r="AQ5" s="63"/>
     </row>
-    <row r="6" spans="1:43" ht="21" x14ac:dyDescent="0.55000000000000004">
+    <row r="6" spans="1:43" ht="19" x14ac:dyDescent="0.25">
       <c r="B6" s="10"/>
       <c r="C6" s="2"/>
       <c r="D6" s="1"/>
@@ -42126,7 +42127,7 @@
       <c r="G6" s="29">
         <v>4</v>
       </c>
-      <c r="H6" s="70" t="s">
+      <c r="H6" s="66" t="s">
         <v>55</v>
       </c>
       <c r="J6" s="10"/>
@@ -42138,7 +42139,7 @@
       <c r="P6" s="29">
         <v>1</v>
       </c>
-      <c r="Q6" s="70" t="s">
+      <c r="Q6" s="66" t="s">
         <v>55</v>
       </c>
       <c r="S6" s="10"/>
@@ -42150,7 +42151,7 @@
       <c r="Y6" s="29">
         <v>3</v>
       </c>
-      <c r="Z6" s="70" t="s">
+      <c r="Z6" s="66" t="s">
         <v>55</v>
       </c>
       <c r="AB6" s="10"/>
@@ -42162,7 +42163,7 @@
       <c r="AH6" s="29">
         <v>3</v>
       </c>
-      <c r="AI6" s="70" t="s">
+      <c r="AI6" s="66" t="s">
         <v>55</v>
       </c>
       <c r="AK6" s="10"/>
@@ -42173,11 +42174,11 @@
       <c r="AP6" s="29">
         <v>2</v>
       </c>
-      <c r="AQ6" s="70" t="s">
+      <c r="AQ6" s="66" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="7" spans="1:43" ht="21" x14ac:dyDescent="0.55000000000000004">
+    <row r="7" spans="1:43" ht="19" x14ac:dyDescent="0.25">
       <c r="B7" s="10"/>
       <c r="C7" s="2"/>
       <c r="D7" s="1"/>
@@ -42186,7 +42187,7 @@
       <c r="G7" s="29">
         <v>7</v>
       </c>
-      <c r="H7" s="70" t="s">
+      <c r="H7" s="66" t="s">
         <v>56</v>
       </c>
       <c r="J7" s="10"/>
@@ -42198,7 +42199,7 @@
       <c r="P7" s="29">
         <v>-2</v>
       </c>
-      <c r="Q7" s="70" t="s">
+      <c r="Q7" s="66" t="s">
         <v>56</v>
       </c>
       <c r="S7" s="10"/>
@@ -42210,7 +42211,7 @@
       <c r="Y7" s="29">
         <v>1</v>
       </c>
-      <c r="Z7" s="70" t="s">
+      <c r="Z7" s="66" t="s">
         <v>56</v>
       </c>
       <c r="AB7" s="10"/>
@@ -42222,7 +42223,7 @@
       <c r="AH7" s="29">
         <v>1</v>
       </c>
-      <c r="AI7" s="70" t="s">
+      <c r="AI7" s="66" t="s">
         <v>56</v>
       </c>
       <c r="AK7" s="10"/>
@@ -42233,16 +42234,16 @@
       <c r="AP7" s="29">
         <v>3</v>
       </c>
-      <c r="AQ7" s="70" t="s">
+      <c r="AQ7" s="66" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="8" spans="1:43" ht="21.4" thickBot="1" x14ac:dyDescent="0.6">
+    <row r="8" spans="1:43" ht="20" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B8" s="10"/>
-      <c r="C8" s="82" t="s">
+      <c r="C8" s="86" t="s">
         <v>47</v>
       </c>
-      <c r="D8" s="82"/>
+      <c r="D8" s="86"/>
       <c r="E8" s="47" t="s">
         <v>48</v>
       </c>
@@ -42250,49 +42251,49 @@
       <c r="G8" s="45">
         <v>1</v>
       </c>
-      <c r="H8" s="84"/>
-      <c r="I8" s="85"/>
-      <c r="J8" s="86"/>
-      <c r="K8" s="85"/>
-      <c r="L8" s="85"/>
-      <c r="M8" s="85"/>
-      <c r="N8" s="85"/>
-      <c r="O8" s="85"/>
+      <c r="H8" s="76"/>
+      <c r="I8" s="77"/>
+      <c r="J8" s="78"/>
+      <c r="K8" s="77"/>
+      <c r="L8" s="77"/>
+      <c r="M8" s="77"/>
+      <c r="N8" s="77"/>
+      <c r="O8" s="77"/>
       <c r="P8" s="29">
         <v>3</v>
       </c>
-      <c r="Q8" s="87" t="s">
+      <c r="Q8" s="79" t="s">
         <v>57</v>
       </c>
-      <c r="S8" s="86"/>
-      <c r="T8" s="85"/>
-      <c r="U8" s="85"/>
-      <c r="V8" s="85"/>
-      <c r="W8" s="85"/>
-      <c r="X8" s="85"/>
+      <c r="S8" s="78"/>
+      <c r="T8" s="77"/>
+      <c r="U8" s="77"/>
+      <c r="V8" s="77"/>
+      <c r="W8" s="77"/>
+      <c r="X8" s="77"/>
       <c r="Y8" s="29">
         <v>2</v>
       </c>
-      <c r="Z8" s="87" t="s">
+      <c r="Z8" s="79" t="s">
         <v>57</v>
       </c>
-      <c r="AB8" s="86"/>
-      <c r="AC8" s="85"/>
-      <c r="AD8" s="85"/>
-      <c r="AE8" s="85"/>
-      <c r="AF8" s="85"/>
-      <c r="AG8" s="85"/>
+      <c r="AB8" s="78"/>
+      <c r="AC8" s="77"/>
+      <c r="AD8" s="77"/>
+      <c r="AE8" s="77"/>
+      <c r="AF8" s="77"/>
+      <c r="AG8" s="77"/>
       <c r="AH8" s="29">
         <v>2</v>
       </c>
-      <c r="AI8" s="87" t="s">
+      <c r="AI8" s="79" t="s">
         <v>57</v>
       </c>
       <c r="AK8" s="10"/>
-      <c r="AL8" s="82" t="s">
+      <c r="AL8" s="86" t="s">
         <v>47</v>
       </c>
-      <c r="AM8" s="82"/>
+      <c r="AM8" s="86"/>
       <c r="AN8" s="47" t="s">
         <v>48</v>
       </c>
@@ -42300,9 +42301,9 @@
       <c r="AP8" s="45">
         <v>1</v>
       </c>
-      <c r="AQ8" s="68"/>
+      <c r="AQ8" s="64"/>
     </row>
-    <row r="9" spans="1:43" ht="21.4" thickBot="1" x14ac:dyDescent="0.6">
+    <row r="9" spans="1:43" ht="20" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B9" s="10"/>
       <c r="C9" s="20">
         <v>1</v>
@@ -42320,16 +42321,16 @@
         <f>C9*G6+D9*G7+E9</f>
         <v>11</v>
       </c>
-      <c r="H9" s="71" t="s">
+      <c r="H9" s="67" t="s">
         <v>52</v>
       </c>
-      <c r="I9" s="85"/>
+      <c r="I9" s="77"/>
       <c r="J9" s="46"/>
-      <c r="K9" s="88" t="s">
+      <c r="K9" s="87" t="s">
         <v>47</v>
       </c>
-      <c r="L9" s="88"/>
-      <c r="M9" s="88"/>
+      <c r="L9" s="87"/>
+      <c r="M9" s="87"/>
       <c r="N9" s="47" t="s">
         <v>48</v>
       </c>
@@ -42337,13 +42338,13 @@
       <c r="P9" s="45">
         <v>1</v>
       </c>
-      <c r="Q9" s="68"/>
+      <c r="Q9" s="64"/>
       <c r="S9" s="46"/>
-      <c r="T9" s="88" t="s">
+      <c r="T9" s="87" t="s">
         <v>47</v>
       </c>
-      <c r="U9" s="88"/>
-      <c r="V9" s="88"/>
+      <c r="U9" s="87"/>
+      <c r="V9" s="87"/>
       <c r="W9" s="47" t="s">
         <v>48</v>
       </c>
@@ -42351,13 +42352,13 @@
       <c r="Y9" s="45">
         <v>1</v>
       </c>
-      <c r="Z9" s="68"/>
+      <c r="Z9" s="64"/>
       <c r="AB9" s="46"/>
-      <c r="AC9" s="88" t="s">
+      <c r="AC9" s="87" t="s">
         <v>47</v>
       </c>
-      <c r="AD9" s="88"/>
-      <c r="AE9" s="88"/>
+      <c r="AD9" s="87"/>
+      <c r="AE9" s="87"/>
       <c r="AF9" s="47" t="s">
         <v>48</v>
       </c>
@@ -42365,7 +42366,7 @@
       <c r="AH9" s="45">
         <v>1</v>
       </c>
-      <c r="AI9" s="68"/>
+      <c r="AI9" s="64"/>
       <c r="AK9" s="10"/>
       <c r="AL9" s="49"/>
       <c r="AM9" s="31">
@@ -42380,12 +42381,12 @@
       <c r="AP9" s="50">
         <v>5</v>
       </c>
-      <c r="AQ9" s="70" t="s">
+      <c r="AQ9" s="66" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="10" spans="1:43" ht="21" x14ac:dyDescent="0.55000000000000004">
-      <c r="B10" s="75"/>
+    <row r="10" spans="1:43" ht="19" x14ac:dyDescent="0.25">
+      <c r="B10" s="68"/>
       <c r="C10" s="25">
         <v>1</v>
       </c>
@@ -42402,7 +42403,7 @@
         <f>C10*G6+D10*G7+E10</f>
         <v>-3</v>
       </c>
-      <c r="H10" s="71" t="s">
+      <c r="H10" s="67" t="s">
         <v>53</v>
       </c>
       <c r="J10" s="10"/>
@@ -42422,7 +42423,7 @@
         <v>43</v>
       </c>
       <c r="P10" s="43"/>
-      <c r="Q10" s="71" t="s">
+      <c r="Q10" s="67" t="s">
         <v>52</v>
       </c>
       <c r="S10" s="10"/>
@@ -42445,7 +42446,7 @@
         <f>T10*Y6+U10*Y7+V10*Y8+W10</f>
         <v>3</v>
       </c>
-      <c r="Z10" s="71" t="s">
+      <c r="Z10" s="67" t="s">
         <v>52</v>
       </c>
       <c r="AB10" s="10"/>
@@ -42468,18 +42469,18 @@
         <f>AC10*AH6+AD10*AH7+AE10*AH8+AF10</f>
         <v>4</v>
       </c>
-      <c r="AI10" s="71" t="s">
+      <c r="AI10" s="67" t="s">
         <v>52</v>
       </c>
-      <c r="AK10" s="75"/>
+      <c r="AK10" s="68"/>
       <c r="AM10" s="1"/>
-      <c r="AN10" s="69"/>
+      <c r="AN10" s="65"/>
       <c r="AO10" s="1"/>
       <c r="AP10" s="1"/>
-      <c r="AQ10" s="67"/>
+      <c r="AQ10" s="63"/>
     </row>
-    <row r="11" spans="1:43" ht="21.4" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="B11" s="76"/>
+    <row r="11" spans="1:43" ht="20" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B11" s="69"/>
       <c r="C11" s="34">
         <v>-1</v>
       </c>
@@ -42493,10 +42494,10 @@
         <v>43</v>
       </c>
       <c r="G11" s="43"/>
-      <c r="H11" s="71" t="s">
+      <c r="H11" s="67" t="s">
         <v>54</v>
       </c>
-      <c r="J11" s="75"/>
+      <c r="J11" s="68"/>
       <c r="K11" s="34">
         <v>1</v>
       </c>
@@ -42516,10 +42517,10 @@
         <f>K11*P6+L11*P7+M11*P8+N11</f>
         <v>2</v>
       </c>
-      <c r="Q11" s="71" t="s">
+      <c r="Q11" s="67" t="s">
         <v>53</v>
       </c>
-      <c r="S11" s="75"/>
+      <c r="S11" s="68"/>
       <c r="T11" s="34">
         <v>1</v>
       </c>
@@ -42536,10 +42537,10 @@
         <v>43</v>
       </c>
       <c r="Y11" s="8"/>
-      <c r="Z11" s="71" t="s">
+      <c r="Z11" s="67" t="s">
         <v>53</v>
       </c>
-      <c r="AB11" s="75"/>
+      <c r="AB11" s="68"/>
       <c r="AC11" s="48">
         <v>0</v>
       </c>
@@ -42556,25 +42557,25 @@
         <v>43</v>
       </c>
       <c r="AH11" s="8"/>
-      <c r="AI11" s="71" t="s">
+      <c r="AI11" s="67" t="s">
         <v>53</v>
       </c>
-      <c r="AK11" s="76"/>
-      <c r="AL11" s="83"/>
+      <c r="AK11" s="69"/>
+      <c r="AL11" s="75"/>
       <c r="AM11" s="1"/>
-      <c r="AN11" s="69"/>
+      <c r="AN11" s="65"/>
       <c r="AO11" s="1"/>
       <c r="AP11" s="1"/>
-      <c r="AQ11" s="77"/>
+      <c r="AQ11" s="70"/>
     </row>
-    <row r="12" spans="1:43" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="B12" s="75"/>
-      <c r="H12" s="67"/>
-      <c r="J12" s="76"/>
-      <c r="Q12" s="67"/>
-      <c r="S12" s="76"/>
-      <c r="Z12" s="67"/>
-      <c r="AB12" s="75"/>
+    <row r="12" spans="1:43" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B12" s="68"/>
+      <c r="H12" s="63"/>
+      <c r="J12" s="69"/>
+      <c r="Q12" s="63"/>
+      <c r="S12" s="69"/>
+      <c r="Z12" s="63"/>
+      <c r="AB12" s="68"/>
       <c r="AC12" s="34">
         <v>1</v>
       </c>
@@ -42594,166 +42595,166 @@
         <f>AC12*AH6+AD12*AH7+AE12*AH8+AF12</f>
         <v>5</v>
       </c>
-      <c r="AI12" s="71" t="s">
+      <c r="AI12" s="67" t="s">
         <v>54</v>
       </c>
       <c r="AK12" s="15"/>
       <c r="AL12" s="1"/>
       <c r="AM12" s="1"/>
-      <c r="AN12" s="69"/>
+      <c r="AN12" s="65"/>
       <c r="AO12" s="1"/>
       <c r="AP12" s="1"/>
-      <c r="AQ12" s="67"/>
+      <c r="AQ12" s="63"/>
     </row>
-    <row r="13" spans="1:43" ht="18" x14ac:dyDescent="0.55000000000000004">
-      <c r="B13" s="75"/>
+    <row r="13" spans="1:43" ht="19" x14ac:dyDescent="0.25">
+      <c r="B13" s="68"/>
       <c r="H13" s="39"/>
-      <c r="J13" s="75"/>
-      <c r="Q13" s="67"/>
-      <c r="S13" s="75"/>
-      <c r="Z13" s="67"/>
-      <c r="AB13" s="75"/>
-      <c r="AI13" s="67"/>
+      <c r="J13" s="68"/>
+      <c r="Q13" s="63"/>
+      <c r="S13" s="68"/>
+      <c r="Z13" s="63"/>
+      <c r="AB13" s="68"/>
+      <c r="AI13" s="63"/>
       <c r="AK13" s="15"/>
       <c r="AL13" s="1"/>
       <c r="AM13" s="1"/>
-      <c r="AN13" s="69"/>
+      <c r="AN13" s="65"/>
       <c r="AO13" s="1"/>
       <c r="AP13" s="1"/>
-      <c r="AQ13" s="67"/>
+      <c r="AQ13" s="63"/>
     </row>
-    <row r="14" spans="1:43" ht="20" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B14" s="75"/>
+    <row r="14" spans="1:43" ht="20" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B14" s="68"/>
       <c r="H14" s="39"/>
-      <c r="J14" s="75"/>
-      <c r="Q14" s="67"/>
-      <c r="S14" s="75"/>
-      <c r="Z14" s="67"/>
-      <c r="AB14" s="75"/>
-      <c r="AI14" s="67"/>
+      <c r="J14" s="68"/>
+      <c r="Q14" s="63"/>
+      <c r="S14" s="68"/>
+      <c r="Z14" s="63"/>
+      <c r="AB14" s="68"/>
+      <c r="AI14" s="63"/>
       <c r="AK14" s="15"/>
       <c r="AL14" s="1"/>
       <c r="AM14" s="1"/>
-      <c r="AN14" s="69"/>
+      <c r="AN14" s="65"/>
       <c r="AO14" s="1"/>
       <c r="AP14" s="1"/>
-      <c r="AQ14" s="67"/>
+      <c r="AQ14" s="63"/>
     </row>
-    <row r="15" spans="1:43" ht="18" x14ac:dyDescent="0.55000000000000004">
-      <c r="B15" s="75"/>
+    <row r="15" spans="1:43" ht="19" x14ac:dyDescent="0.25">
+      <c r="B15" s="68"/>
       <c r="H15" s="39"/>
-      <c r="J15" s="75"/>
-      <c r="Q15" s="67"/>
-      <c r="S15" s="75"/>
-      <c r="Z15" s="67"/>
-      <c r="AB15" s="75"/>
-      <c r="AI15" s="67"/>
+      <c r="J15" s="68"/>
+      <c r="Q15" s="63"/>
+      <c r="S15" s="68"/>
+      <c r="Z15" s="63"/>
+      <c r="AB15" s="68"/>
+      <c r="AI15" s="63"/>
       <c r="AK15" s="15"/>
       <c r="AL15" s="1"/>
-      <c r="AQ15" s="67"/>
+      <c r="AQ15" s="63"/>
     </row>
-    <row r="16" spans="1:43" ht="21" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B16" s="75"/>
+    <row r="16" spans="1:43" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B16" s="68"/>
       <c r="H16" s="39"/>
-      <c r="J16" s="75"/>
-      <c r="Q16" s="67"/>
-      <c r="S16" s="75"/>
-      <c r="Z16" s="67"/>
-      <c r="AB16" s="75"/>
-      <c r="AI16" s="67"/>
+      <c r="J16" s="68"/>
+      <c r="Q16" s="63"/>
+      <c r="S16" s="68"/>
+      <c r="Z16" s="63"/>
+      <c r="AB16" s="68"/>
+      <c r="AI16" s="63"/>
       <c r="AK16" s="15"/>
       <c r="AL16" s="1"/>
-      <c r="AQ16" s="67"/>
+      <c r="AQ16" s="63"/>
     </row>
-    <row r="17" spans="2:43" ht="19.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B17" s="75"/>
-      <c r="H17" s="67"/>
-      <c r="J17" s="75"/>
-      <c r="Q17" s="67"/>
-      <c r="S17" s="75"/>
-      <c r="Z17" s="67"/>
-      <c r="AB17" s="75"/>
-      <c r="AI17" s="67"/>
+    <row r="17" spans="2:43" ht="19" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B17" s="68"/>
+      <c r="H17" s="63"/>
+      <c r="J17" s="68"/>
+      <c r="Q17" s="63"/>
+      <c r="S17" s="68"/>
+      <c r="Z17" s="63"/>
+      <c r="AB17" s="68"/>
+      <c r="AI17" s="63"/>
       <c r="AK17" s="15"/>
       <c r="AL17" s="1"/>
-      <c r="AQ17" s="67"/>
+      <c r="AQ17" s="63"/>
     </row>
-    <row r="18" spans="2:43" ht="19.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B18" s="75"/>
-      <c r="H18" s="67"/>
-      <c r="J18" s="75"/>
-      <c r="Q18" s="67"/>
-      <c r="S18" s="75"/>
-      <c r="Z18" s="67"/>
-      <c r="AB18" s="75"/>
-      <c r="AI18" s="67"/>
+    <row r="18" spans="2:43" ht="19" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B18" s="68"/>
+      <c r="H18" s="63"/>
+      <c r="J18" s="68"/>
+      <c r="Q18" s="63"/>
+      <c r="S18" s="68"/>
+      <c r="Z18" s="63"/>
+      <c r="AB18" s="68"/>
+      <c r="AI18" s="63"/>
       <c r="AK18" s="15"/>
       <c r="AL18" s="1"/>
       <c r="AM18" s="2"/>
       <c r="AN18" s="2"/>
       <c r="AO18" s="2"/>
       <c r="AP18" s="2"/>
-      <c r="AQ18" s="67"/>
+      <c r="AQ18" s="63"/>
     </row>
-    <row r="19" spans="2:43" ht="19.05" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="B19" s="75"/>
-      <c r="H19" s="67"/>
-      <c r="J19" s="75"/>
-      <c r="Q19" s="67"/>
-      <c r="S19" s="75"/>
-      <c r="Z19" s="67"/>
-      <c r="AB19" s="75"/>
-      <c r="AI19" s="67"/>
+    <row r="19" spans="2:43" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B19" s="68"/>
+      <c r="H19" s="63"/>
+      <c r="J19" s="68"/>
+      <c r="Q19" s="63"/>
+      <c r="S19" s="68"/>
+      <c r="Z19" s="63"/>
+      <c r="AB19" s="68"/>
+      <c r="AI19" s="63"/>
       <c r="AK19" s="11"/>
       <c r="AL19" s="12"/>
-      <c r="AM19" s="79"/>
-      <c r="AN19" s="79"/>
-      <c r="AO19" s="79"/>
-      <c r="AP19" s="79"/>
-      <c r="AQ19" s="78"/>
+      <c r="AM19" s="72"/>
+      <c r="AN19" s="72"/>
+      <c r="AO19" s="72"/>
+      <c r="AP19" s="72"/>
+      <c r="AQ19" s="71"/>
     </row>
-    <row r="20" spans="2:43" ht="20" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B20" s="75"/>
+    <row r="20" spans="2:43" ht="20" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B20" s="68"/>
       <c r="H20" s="40"/>
-      <c r="J20" s="75"/>
-      <c r="Q20" s="67"/>
-      <c r="S20" s="75"/>
-      <c r="Z20" s="67"/>
-      <c r="AB20" s="75"/>
-      <c r="AI20" s="67"/>
+      <c r="J20" s="68"/>
+      <c r="Q20" s="63"/>
+      <c r="S20" s="68"/>
+      <c r="Z20" s="63"/>
+      <c r="AB20" s="68"/>
+      <c r="AI20" s="63"/>
     </row>
-    <row r="21" spans="2:43" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B21" s="80"/>
-      <c r="C21" s="79"/>
-      <c r="D21" s="79"/>
-      <c r="E21" s="79"/>
-      <c r="F21" s="79"/>
-      <c r="G21" s="79"/>
-      <c r="H21" s="78"/>
-      <c r="J21" s="80"/>
-      <c r="K21" s="79"/>
-      <c r="L21" s="79"/>
-      <c r="M21" s="79"/>
-      <c r="N21" s="79"/>
-      <c r="O21" s="79"/>
-      <c r="P21" s="79"/>
-      <c r="Q21" s="78"/>
-      <c r="S21" s="80"/>
-      <c r="T21" s="79"/>
-      <c r="U21" s="79"/>
-      <c r="V21" s="79"/>
-      <c r="W21" s="79"/>
-      <c r="X21" s="79"/>
-      <c r="Y21" s="79"/>
-      <c r="Z21" s="78"/>
-      <c r="AB21" s="80"/>
-      <c r="AC21" s="79"/>
-      <c r="AD21" s="79"/>
-      <c r="AE21" s="79"/>
-      <c r="AF21" s="79"/>
-      <c r="AG21" s="79"/>
-      <c r="AH21" s="79"/>
-      <c r="AI21" s="78"/>
+    <row r="21" spans="2:43" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B21" s="73"/>
+      <c r="C21" s="72"/>
+      <c r="D21" s="72"/>
+      <c r="E21" s="72"/>
+      <c r="F21" s="72"/>
+      <c r="G21" s="72"/>
+      <c r="H21" s="71"/>
+      <c r="J21" s="73"/>
+      <c r="K21" s="72"/>
+      <c r="L21" s="72"/>
+      <c r="M21" s="72"/>
+      <c r="N21" s="72"/>
+      <c r="O21" s="72"/>
+      <c r="P21" s="72"/>
+      <c r="Q21" s="71"/>
+      <c r="S21" s="73"/>
+      <c r="T21" s="72"/>
+      <c r="U21" s="72"/>
+      <c r="V21" s="72"/>
+      <c r="W21" s="72"/>
+      <c r="X21" s="72"/>
+      <c r="Y21" s="72"/>
+      <c r="Z21" s="71"/>
+      <c r="AB21" s="73"/>
+      <c r="AC21" s="72"/>
+      <c r="AD21" s="72"/>
+      <c r="AE21" s="72"/>
+      <c r="AF21" s="72"/>
+      <c r="AG21" s="72"/>
+      <c r="AH21" s="72"/>
+      <c r="AI21" s="71"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -42779,50 +42780,46 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{688B5BB5-4F72-764D-85DB-452B7F72780F}">
   <dimension ref="A1:AN20"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.5"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="11" style="63"/>
-    <col min="2" max="2" width="4.6875" style="63" customWidth="1"/>
-    <col min="3" max="3" width="4.8125" style="63" customWidth="1"/>
-    <col min="4" max="5" width="4.6875" style="63" customWidth="1"/>
-    <col min="6" max="6" width="5" style="63" customWidth="1"/>
-    <col min="7" max="7" width="4.5" style="63" customWidth="1"/>
-    <col min="8" max="8" width="4.3125" style="63" customWidth="1"/>
-    <col min="9" max="9" width="10.5" style="63" customWidth="1"/>
-    <col min="10" max="10" width="4.8125" style="63" customWidth="1"/>
-    <col min="11" max="11" width="5" style="63" customWidth="1"/>
-    <col min="12" max="12" width="4.5" style="63" customWidth="1"/>
-    <col min="13" max="13" width="4.6875" style="63" customWidth="1"/>
-    <col min="14" max="15" width="4.8125" style="63" customWidth="1"/>
-    <col min="16" max="16" width="5" style="63" customWidth="1"/>
-    <col min="17" max="17" width="9.5" style="63" customWidth="1"/>
-    <col min="18" max="18" width="4.8125" style="63" customWidth="1"/>
-    <col min="19" max="19" width="5.1875" style="63" customWidth="1"/>
-    <col min="20" max="20" width="4.6875" style="63" customWidth="1"/>
-    <col min="21" max="21" width="5.1875" style="63" customWidth="1"/>
-    <col min="22" max="22" width="5" style="63" customWidth="1"/>
-    <col min="23" max="23" width="4.8125" style="63" customWidth="1"/>
-    <col min="24" max="24" width="5" style="63" customWidth="1"/>
-    <col min="25" max="25" width="11" style="63"/>
-    <col min="26" max="26" width="5" style="63" customWidth="1"/>
-    <col min="27" max="27" width="5.1875" style="63" customWidth="1"/>
-    <col min="28" max="28" width="5" style="63" customWidth="1"/>
-    <col min="29" max="29" width="4.8125" style="63" customWidth="1"/>
-    <col min="30" max="30" width="5.1875" style="63" customWidth="1"/>
-    <col min="31" max="31" width="4.8125" style="63" customWidth="1"/>
-    <col min="32" max="32" width="5" style="63" customWidth="1"/>
-    <col min="33" max="33" width="11" style="63"/>
-    <col min="34" max="34" width="5.1875" style="63" customWidth="1"/>
-    <col min="35" max="35" width="5.8125" style="63" customWidth="1"/>
-    <col min="36" max="36" width="5.3125" style="63" customWidth="1"/>
-    <col min="37" max="37" width="5.1875" style="63" customWidth="1"/>
-    <col min="38" max="38" width="5" style="63" customWidth="1"/>
-    <col min="39" max="39" width="4.8125" style="63" customWidth="1"/>
-    <col min="40" max="40" width="5.3125" style="63" customWidth="1"/>
-    <col min="41" max="16384" width="11" style="63"/>
+    <col min="2" max="2" width="4.6640625" customWidth="1"/>
+    <col min="3" max="3" width="4.83203125" customWidth="1"/>
+    <col min="4" max="5" width="4.6640625" customWidth="1"/>
+    <col min="6" max="6" width="5" customWidth="1"/>
+    <col min="7" max="7" width="4.5" customWidth="1"/>
+    <col min="8" max="8" width="4.33203125" customWidth="1"/>
+    <col min="9" max="9" width="10.5" customWidth="1"/>
+    <col min="10" max="10" width="4.83203125" customWidth="1"/>
+    <col min="11" max="11" width="5" customWidth="1"/>
+    <col min="12" max="12" width="4.5" customWidth="1"/>
+    <col min="13" max="13" width="4.6640625" customWidth="1"/>
+    <col min="14" max="15" width="4.83203125" customWidth="1"/>
+    <col min="16" max="16" width="5" customWidth="1"/>
+    <col min="17" max="17" width="9.5" customWidth="1"/>
+    <col min="18" max="18" width="4.83203125" customWidth="1"/>
+    <col min="19" max="19" width="5.1640625" customWidth="1"/>
+    <col min="20" max="20" width="4.6640625" customWidth="1"/>
+    <col min="21" max="21" width="5.1640625" customWidth="1"/>
+    <col min="22" max="22" width="5" customWidth="1"/>
+    <col min="23" max="23" width="4.83203125" customWidth="1"/>
+    <col min="24" max="24" width="5" customWidth="1"/>
+    <col min="26" max="26" width="5" customWidth="1"/>
+    <col min="27" max="27" width="5.1640625" customWidth="1"/>
+    <col min="28" max="28" width="5" customWidth="1"/>
+    <col min="29" max="29" width="4.83203125" customWidth="1"/>
+    <col min="30" max="30" width="5.1640625" customWidth="1"/>
+    <col min="31" max="31" width="4.83203125" customWidth="1"/>
+    <col min="32" max="32" width="5" customWidth="1"/>
+    <col min="34" max="34" width="5.1640625" customWidth="1"/>
+    <col min="35" max="35" width="5.83203125" customWidth="1"/>
+    <col min="36" max="36" width="5.33203125" customWidth="1"/>
+    <col min="37" max="37" width="5.1640625" customWidth="1"/>
+    <col min="38" max="38" width="5" customWidth="1"/>
+    <col min="39" max="39" width="4.83203125" customWidth="1"/>
+    <col min="40" max="40" width="5.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:40" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:40" s="2" customFormat="1" ht="19" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>51</v>
       </c>
@@ -42838,11 +42835,11 @@
       <c r="O1" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="R1" s="81" t="s">
+      <c r="R1" s="74" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="3" spans="1:40" ht="18.399999999999999" thickBot="1" x14ac:dyDescent="0.6">
+    <row r="3" spans="1:40" ht="20" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="2" t="str">
         <f>IF(ISBLANK(D9)=TRUE,"NOT DONE",IF(B5=D9,"CORRECT", "INCORRECT"))</f>
         <v>NOT DONE</v>
@@ -42889,54 +42886,54 @@
       <c r="AL3" s="2"/>
       <c r="AM3" s="2"/>
     </row>
-    <row r="4" spans="1:40" ht="18" x14ac:dyDescent="0.55000000000000004">
-      <c r="B4" s="64" t="s">
+    <row r="4" spans="1:40" ht="19" x14ac:dyDescent="0.25">
+      <c r="B4" s="80" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="65"/>
-      <c r="D4" s="65"/>
-      <c r="E4" s="65"/>
-      <c r="F4" s="65"/>
-      <c r="G4" s="65"/>
-      <c r="H4" s="66"/>
-      <c r="J4" s="64" t="s">
+      <c r="C4" s="81"/>
+      <c r="D4" s="81"/>
+      <c r="E4" s="81"/>
+      <c r="F4" s="81"/>
+      <c r="G4" s="81"/>
+      <c r="H4" s="82"/>
+      <c r="J4" s="80" t="s">
         <v>16</v>
       </c>
-      <c r="K4" s="65"/>
-      <c r="L4" s="65"/>
-      <c r="M4" s="65"/>
-      <c r="N4" s="65"/>
-      <c r="O4" s="65"/>
-      <c r="P4" s="66"/>
-      <c r="R4" s="64" t="s">
+      <c r="K4" s="81"/>
+      <c r="L4" s="81"/>
+      <c r="M4" s="81"/>
+      <c r="N4" s="81"/>
+      <c r="O4" s="81"/>
+      <c r="P4" s="82"/>
+      <c r="R4" s="80" t="s">
         <v>17</v>
       </c>
-      <c r="S4" s="65"/>
-      <c r="T4" s="65"/>
-      <c r="U4" s="65"/>
-      <c r="V4" s="65"/>
-      <c r="W4" s="65"/>
-      <c r="X4" s="66"/>
-      <c r="Z4" s="64" t="s">
+      <c r="S4" s="81"/>
+      <c r="T4" s="81"/>
+      <c r="U4" s="81"/>
+      <c r="V4" s="81"/>
+      <c r="W4" s="81"/>
+      <c r="X4" s="82"/>
+      <c r="Z4" s="80" t="s">
         <v>18</v>
       </c>
-      <c r="AA4" s="65"/>
-      <c r="AB4" s="65"/>
-      <c r="AC4" s="65"/>
-      <c r="AD4" s="65"/>
-      <c r="AE4" s="65"/>
-      <c r="AF4" s="66"/>
-      <c r="AH4" s="64" t="s">
+      <c r="AA4" s="81"/>
+      <c r="AB4" s="81"/>
+      <c r="AC4" s="81"/>
+      <c r="AD4" s="81"/>
+      <c r="AE4" s="81"/>
+      <c r="AF4" s="82"/>
+      <c r="AH4" s="80" t="s">
         <v>19</v>
       </c>
-      <c r="AI4" s="65"/>
-      <c r="AJ4" s="65"/>
-      <c r="AK4" s="65"/>
-      <c r="AL4" s="65"/>
-      <c r="AM4" s="65"/>
-      <c r="AN4" s="66"/>
+      <c r="AI4" s="81"/>
+      <c r="AJ4" s="81"/>
+      <c r="AK4" s="81"/>
+      <c r="AL4" s="81"/>
+      <c r="AM4" s="81"/>
+      <c r="AN4" s="82"/>
     </row>
-    <row r="5" spans="1:40" ht="18" x14ac:dyDescent="0.55000000000000004">
+    <row r="5" spans="1:40" ht="19" x14ac:dyDescent="0.25">
       <c r="B5" s="14">
         <f>(G9-E9-G6*C9)/G7</f>
         <v>0</v>
@@ -42946,7 +42943,7 @@
       <c r="E5" s="2"/>
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
-      <c r="H5" s="67"/>
+      <c r="H5" s="63"/>
       <c r="J5" s="14">
         <f>O9-O6*K9-O7*L9</f>
         <v>2</v>
@@ -42956,7 +42953,7 @@
       <c r="M5" s="2"/>
       <c r="N5" s="2"/>
       <c r="O5" s="2"/>
-      <c r="P5" s="67"/>
+      <c r="P5" s="63"/>
       <c r="R5" s="14">
         <f>W9-W6*S9-W7*T9</f>
         <v>-2</v>
@@ -42966,7 +42963,7 @@
       <c r="U5" s="2"/>
       <c r="V5" s="2"/>
       <c r="W5" s="2"/>
-      <c r="X5" s="67"/>
+      <c r="X5" s="63"/>
       <c r="Z5" s="14">
         <f>(AE9-AC9-AE7*AB9)/AE6</f>
         <v>-1</v>
@@ -42976,7 +42973,7 @@
       <c r="AC5" s="2"/>
       <c r="AD5" s="2"/>
       <c r="AE5" s="2"/>
-      <c r="AF5" s="67"/>
+      <c r="AF5" s="63"/>
       <c r="AH5" s="9">
         <f>(AM10-AK10-AM6*AI10)/AM7</f>
         <v>3</v>
@@ -42986,9 +42983,9 @@
       <c r="AK5" s="2"/>
       <c r="AL5" s="2"/>
       <c r="AM5" s="2"/>
-      <c r="AN5" s="67"/>
+      <c r="AN5" s="63"/>
     </row>
-    <row r="6" spans="1:40" ht="21" x14ac:dyDescent="0.55000000000000004">
+    <row r="6" spans="1:40" ht="19" x14ac:dyDescent="0.25">
       <c r="B6" s="10"/>
       <c r="C6" s="2"/>
       <c r="D6" s="1"/>
@@ -42997,7 +42994,7 @@
       <c r="G6" s="29">
         <v>2</v>
       </c>
-      <c r="H6" s="70" t="s">
+      <c r="H6" s="66" t="s">
         <v>55</v>
       </c>
       <c r="J6" s="10"/>
@@ -43008,7 +43005,7 @@
       <c r="O6" s="29">
         <v>2</v>
       </c>
-      <c r="P6" s="70" t="s">
+      <c r="P6" s="66" t="s">
         <v>55</v>
       </c>
       <c r="R6" s="10"/>
@@ -43019,7 +43016,7 @@
       <c r="W6" s="29">
         <v>2</v>
       </c>
-      <c r="X6" s="70" t="s">
+      <c r="X6" s="66" t="s">
         <v>55</v>
       </c>
       <c r="Z6" s="10"/>
@@ -43030,7 +43027,7 @@
       <c r="AE6" s="29">
         <v>3</v>
       </c>
-      <c r="AF6" s="70" t="s">
+      <c r="AF6" s="66" t="s">
         <v>55</v>
       </c>
       <c r="AH6" s="10"/>
@@ -43041,11 +43038,11 @@
       <c r="AM6" s="29">
         <v>4</v>
       </c>
-      <c r="AN6" s="70" t="s">
+      <c r="AN6" s="66" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="7" spans="1:40" ht="21" x14ac:dyDescent="0.55000000000000004">
+    <row r="7" spans="1:40" ht="19" x14ac:dyDescent="0.25">
       <c r="B7" s="10"/>
       <c r="C7" s="2"/>
       <c r="D7" s="1"/>
@@ -43054,7 +43051,7 @@
       <c r="G7" s="29">
         <v>3</v>
       </c>
-      <c r="H7" s="70" t="s">
+      <c r="H7" s="66" t="s">
         <v>56</v>
       </c>
       <c r="J7" s="10"/>
@@ -43065,7 +43062,7 @@
       <c r="O7" s="29">
         <v>1</v>
       </c>
-      <c r="P7" s="70" t="s">
+      <c r="P7" s="66" t="s">
         <v>56</v>
       </c>
       <c r="R7" s="10"/>
@@ -43076,7 +43073,7 @@
       <c r="W7" s="29">
         <v>1</v>
       </c>
-      <c r="X7" s="70" t="s">
+      <c r="X7" s="66" t="s">
         <v>56</v>
       </c>
       <c r="Z7" s="10"/>
@@ -43087,7 +43084,7 @@
       <c r="AE7" s="29">
         <v>5</v>
       </c>
-      <c r="AF7" s="70" t="s">
+      <c r="AF7" s="66" t="s">
         <v>56</v>
       </c>
       <c r="AH7" s="10"/>
@@ -43098,16 +43095,16 @@
       <c r="AM7" s="29">
         <v>2</v>
       </c>
-      <c r="AN7" s="70" t="s">
+      <c r="AN7" s="66" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="8" spans="1:40" ht="18.399999999999999" thickBot="1" x14ac:dyDescent="0.6">
+    <row r="8" spans="1:40" ht="20" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B8" s="10"/>
-      <c r="C8" s="82" t="s">
+      <c r="C8" s="86" t="s">
         <v>47</v>
       </c>
-      <c r="D8" s="82"/>
+      <c r="D8" s="86"/>
       <c r="E8" s="47" t="s">
         <v>48</v>
       </c>
@@ -43115,12 +43112,12 @@
       <c r="G8" s="45">
         <v>1</v>
       </c>
-      <c r="H8" s="68"/>
+      <c r="H8" s="64"/>
       <c r="J8" s="10"/>
-      <c r="K8" s="82" t="s">
+      <c r="K8" s="86" t="s">
         <v>47</v>
       </c>
-      <c r="L8" s="82"/>
+      <c r="L8" s="86"/>
       <c r="M8" s="47" t="s">
         <v>48</v>
       </c>
@@ -43128,12 +43125,12 @@
       <c r="O8" s="45">
         <v>1</v>
       </c>
-      <c r="P8" s="68"/>
+      <c r="P8" s="64"/>
       <c r="R8" s="10"/>
-      <c r="S8" s="82" t="s">
+      <c r="S8" s="86" t="s">
         <v>47</v>
       </c>
-      <c r="T8" s="82"/>
+      <c r="T8" s="86"/>
       <c r="U8" s="47" t="s">
         <v>48</v>
       </c>
@@ -43141,12 +43138,12 @@
       <c r="W8" s="45">
         <v>1</v>
       </c>
-      <c r="X8" s="68"/>
+      <c r="X8" s="64"/>
       <c r="Z8" s="10"/>
-      <c r="AA8" s="82" t="s">
+      <c r="AA8" s="86" t="s">
         <v>47</v>
       </c>
-      <c r="AB8" s="82"/>
+      <c r="AB8" s="86"/>
       <c r="AC8" s="47" t="s">
         <v>48</v>
       </c>
@@ -43154,12 +43151,12 @@
       <c r="AE8" s="17">
         <v>1</v>
       </c>
-      <c r="AF8" s="68"/>
+      <c r="AF8" s="64"/>
       <c r="AH8" s="10"/>
-      <c r="AI8" s="82" t="s">
+      <c r="AI8" s="86" t="s">
         <v>47</v>
       </c>
-      <c r="AJ8" s="82"/>
+      <c r="AJ8" s="86"/>
       <c r="AK8" s="47" t="s">
         <v>48</v>
       </c>
@@ -43167,9 +43164,9 @@
       <c r="AM8" s="17">
         <v>1</v>
       </c>
-      <c r="AN8" s="68"/>
+      <c r="AN8" s="64"/>
     </row>
-    <row r="9" spans="1:40" ht="21.4" thickBot="1" x14ac:dyDescent="0.6">
+    <row r="9" spans="1:40" ht="20" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B9" s="10"/>
       <c r="C9" s="30">
         <v>1</v>
@@ -43184,7 +43181,7 @@
       <c r="G9" s="53">
         <v>2</v>
       </c>
-      <c r="H9" s="70" t="s">
+      <c r="H9" s="66" t="s">
         <v>49</v>
       </c>
       <c r="J9" s="10"/>
@@ -43201,7 +43198,7 @@
       <c r="O9" s="53">
         <v>5</v>
       </c>
-      <c r="P9" s="70" t="s">
+      <c r="P9" s="66" t="s">
         <v>49</v>
       </c>
       <c r="R9" s="10"/>
@@ -43218,7 +43215,7 @@
       <c r="W9" s="53">
         <v>1</v>
       </c>
-      <c r="X9" s="70" t="s">
+      <c r="X9" s="66" t="s">
         <v>49</v>
       </c>
       <c r="Z9" s="10"/>
@@ -43235,7 +43232,7 @@
       <c r="AE9" s="42">
         <v>2</v>
       </c>
-      <c r="AF9" s="71" t="s">
+      <c r="AF9" s="67" t="s">
         <v>52</v>
       </c>
       <c r="AH9" s="10"/>
@@ -43255,30 +43252,30 @@
         <f>AI9*AM6+AJ9*AM7+AK9</f>
         <v>8</v>
       </c>
-      <c r="AN9" s="71" t="s">
+      <c r="AN9" s="67" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="10" spans="1:40" ht="21.4" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="B10" s="75"/>
+    <row r="10" spans="1:40" ht="20" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B10" s="68"/>
       <c r="D10" s="1"/>
-      <c r="E10" s="69"/>
+      <c r="E10" s="65"/>
       <c r="F10" s="1"/>
       <c r="G10" s="1"/>
-      <c r="H10" s="67"/>
-      <c r="J10" s="75"/>
+      <c r="H10" s="63"/>
+      <c r="J10" s="68"/>
       <c r="L10" s="1"/>
-      <c r="M10" s="69"/>
+      <c r="M10" s="65"/>
       <c r="N10" s="1"/>
       <c r="O10" s="1"/>
-      <c r="P10" s="67"/>
-      <c r="R10" s="75"/>
+      <c r="P10" s="63"/>
+      <c r="R10" s="68"/>
       <c r="T10" s="1"/>
-      <c r="U10" s="69"/>
+      <c r="U10" s="65"/>
       <c r="V10" s="1"/>
       <c r="W10" s="1"/>
-      <c r="X10" s="67"/>
-      <c r="Z10" s="75"/>
+      <c r="X10" s="63"/>
+      <c r="Z10" s="68"/>
       <c r="AA10" s="22">
         <v>1</v>
       </c>
@@ -43295,10 +43292,10 @@
         <f>AA10*AE6+AB10*AE7+AC10</f>
         <v>-2</v>
       </c>
-      <c r="AF10" s="71" t="s">
+      <c r="AF10" s="67" t="s">
         <v>53</v>
       </c>
-      <c r="AH10" s="75"/>
+      <c r="AH10" s="68"/>
       <c r="AI10" s="34">
         <v>1</v>
       </c>
@@ -43312,272 +43309,272 @@
       <c r="AM10" s="44">
         <v>10</v>
       </c>
-      <c r="AN10" s="71" t="s">
+      <c r="AN10" s="67" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="11" spans="1:40" ht="18" x14ac:dyDescent="0.55000000000000004">
-      <c r="B11" s="76"/>
-      <c r="C11" s="83"/>
+    <row r="11" spans="1:40" ht="19" x14ac:dyDescent="0.25">
+      <c r="B11" s="69"/>
+      <c r="C11" s="75"/>
       <c r="D11" s="1"/>
-      <c r="E11" s="69"/>
+      <c r="E11" s="65"/>
       <c r="F11" s="1"/>
       <c r="G11" s="1"/>
-      <c r="H11" s="77"/>
-      <c r="J11" s="76"/>
-      <c r="K11" s="83"/>
+      <c r="H11" s="70"/>
+      <c r="J11" s="69"/>
+      <c r="K11" s="75"/>
       <c r="L11" s="1"/>
-      <c r="M11" s="69"/>
+      <c r="M11" s="65"/>
       <c r="N11" s="1"/>
       <c r="O11" s="1"/>
-      <c r="P11" s="77"/>
-      <c r="R11" s="76"/>
-      <c r="S11" s="83"/>
+      <c r="P11" s="70"/>
+      <c r="R11" s="69"/>
+      <c r="S11" s="75"/>
       <c r="T11" s="1"/>
-      <c r="U11" s="69"/>
+      <c r="U11" s="65"/>
       <c r="V11" s="1"/>
       <c r="W11" s="1"/>
-      <c r="X11" s="77"/>
-      <c r="Z11" s="76"/>
-      <c r="AF11" s="77"/>
-      <c r="AH11" s="76"/>
-      <c r="AN11" s="77"/>
+      <c r="X11" s="70"/>
+      <c r="Z11" s="69"/>
+      <c r="AF11" s="70"/>
+      <c r="AH11" s="69"/>
+      <c r="AN11" s="70"/>
     </row>
-    <row r="12" spans="1:40" ht="18" x14ac:dyDescent="0.55000000000000004">
+    <row r="12" spans="1:40" ht="19" x14ac:dyDescent="0.25">
       <c r="B12" s="15"/>
       <c r="C12" s="1"/>
       <c r="D12" s="1"/>
-      <c r="E12" s="69"/>
+      <c r="E12" s="65"/>
       <c r="F12" s="1"/>
       <c r="G12" s="1"/>
-      <c r="H12" s="67"/>
+      <c r="H12" s="63"/>
       <c r="J12" s="15"/>
       <c r="K12" s="1"/>
       <c r="L12" s="1"/>
-      <c r="M12" s="69"/>
+      <c r="M12" s="65"/>
       <c r="N12" s="1"/>
       <c r="O12" s="1"/>
-      <c r="P12" s="67"/>
+      <c r="P12" s="63"/>
       <c r="R12" s="15"/>
       <c r="S12" s="1"/>
       <c r="T12" s="1"/>
-      <c r="U12" s="69"/>
+      <c r="U12" s="65"/>
       <c r="V12" s="1"/>
       <c r="W12" s="1"/>
-      <c r="X12" s="67"/>
-      <c r="Z12" s="75"/>
+      <c r="X12" s="63"/>
+      <c r="Z12" s="68"/>
       <c r="AA12" s="1"/>
-      <c r="AB12" s="83"/>
+      <c r="AB12" s="75"/>
       <c r="AC12" s="1"/>
-      <c r="AD12" s="69"/>
+      <c r="AD12" s="65"/>
       <c r="AE12" s="1"/>
       <c r="AF12" s="39"/>
-      <c r="AH12" s="75"/>
+      <c r="AH12" s="68"/>
       <c r="AI12" s="1"/>
-      <c r="AJ12" s="83"/>
+      <c r="AJ12" s="75"/>
       <c r="AK12" s="1"/>
-      <c r="AL12" s="69"/>
+      <c r="AL12" s="65"/>
       <c r="AM12" s="1"/>
       <c r="AN12" s="39"/>
     </row>
-    <row r="13" spans="1:40" ht="18" x14ac:dyDescent="0.55000000000000004">
+    <row r="13" spans="1:40" ht="19" x14ac:dyDescent="0.25">
       <c r="B13" s="15"/>
       <c r="C13" s="1"/>
       <c r="D13" s="1"/>
-      <c r="E13" s="69"/>
+      <c r="E13" s="65"/>
       <c r="F13" s="1"/>
       <c r="G13" s="1"/>
-      <c r="H13" s="67"/>
+      <c r="H13" s="63"/>
       <c r="J13" s="15"/>
       <c r="K13" s="1"/>
       <c r="L13" s="1"/>
-      <c r="M13" s="69"/>
+      <c r="M13" s="65"/>
       <c r="N13" s="1"/>
       <c r="O13" s="1"/>
-      <c r="P13" s="67"/>
+      <c r="P13" s="63"/>
       <c r="R13" s="15"/>
       <c r="S13" s="1"/>
       <c r="T13" s="1"/>
-      <c r="U13" s="69"/>
+      <c r="U13" s="65"/>
       <c r="V13" s="1"/>
       <c r="W13" s="1"/>
-      <c r="X13" s="67"/>
-      <c r="Z13" s="75"/>
+      <c r="X13" s="63"/>
+      <c r="Z13" s="68"/>
       <c r="AA13" s="1"/>
       <c r="AB13" s="1"/>
       <c r="AC13" s="1"/>
-      <c r="AD13" s="69"/>
+      <c r="AD13" s="65"/>
       <c r="AE13" s="1"/>
       <c r="AF13" s="39"/>
-      <c r="AH13" s="75"/>
+      <c r="AH13" s="68"/>
       <c r="AI13" s="1"/>
       <c r="AJ13" s="1"/>
       <c r="AK13" s="1"/>
-      <c r="AL13" s="69"/>
+      <c r="AL13" s="65"/>
       <c r="AM13" s="1"/>
       <c r="AN13" s="39"/>
     </row>
-    <row r="14" spans="1:40" ht="18" x14ac:dyDescent="0.55000000000000004">
+    <row r="14" spans="1:40" ht="19" x14ac:dyDescent="0.25">
       <c r="B14" s="15"/>
       <c r="C14" s="1"/>
       <c r="D14" s="1"/>
-      <c r="E14" s="69"/>
+      <c r="E14" s="65"/>
       <c r="F14" s="1"/>
       <c r="G14" s="1"/>
-      <c r="H14" s="67"/>
+      <c r="H14" s="63"/>
       <c r="J14" s="15"/>
       <c r="K14" s="1"/>
       <c r="L14" s="1"/>
-      <c r="M14" s="69"/>
+      <c r="M14" s="65"/>
       <c r="N14" s="1"/>
       <c r="O14" s="1"/>
-      <c r="P14" s="67"/>
+      <c r="P14" s="63"/>
       <c r="R14" s="15"/>
       <c r="S14" s="1"/>
       <c r="T14" s="1"/>
-      <c r="U14" s="69"/>
+      <c r="U14" s="65"/>
       <c r="V14" s="1"/>
       <c r="W14" s="1"/>
-      <c r="X14" s="67"/>
-      <c r="Z14" s="75"/>
+      <c r="X14" s="63"/>
+      <c r="Z14" s="68"/>
       <c r="AA14" s="1"/>
       <c r="AB14" s="1"/>
       <c r="AC14" s="1"/>
-      <c r="AD14" s="69"/>
+      <c r="AD14" s="65"/>
       <c r="AE14" s="1"/>
       <c r="AF14" s="39"/>
-      <c r="AH14" s="75"/>
+      <c r="AH14" s="68"/>
       <c r="AI14" s="1"/>
       <c r="AJ14" s="1"/>
       <c r="AK14" s="1"/>
-      <c r="AL14" s="69"/>
+      <c r="AL14" s="65"/>
       <c r="AM14" s="1"/>
       <c r="AN14" s="39"/>
     </row>
-    <row r="15" spans="1:40" ht="18" x14ac:dyDescent="0.55000000000000004">
+    <row r="15" spans="1:40" ht="19" x14ac:dyDescent="0.25">
       <c r="B15" s="15"/>
       <c r="C15" s="1"/>
-      <c r="H15" s="67"/>
+      <c r="H15" s="63"/>
       <c r="J15" s="15"/>
       <c r="K15" s="1"/>
-      <c r="P15" s="67"/>
+      <c r="P15" s="63"/>
       <c r="R15" s="15"/>
       <c r="S15" s="1"/>
-      <c r="X15" s="67"/>
-      <c r="Z15" s="75"/>
+      <c r="X15" s="63"/>
+      <c r="Z15" s="68"/>
       <c r="AA15" s="1"/>
       <c r="AB15" s="1"/>
       <c r="AC15" s="1"/>
-      <c r="AD15" s="69"/>
+      <c r="AD15" s="65"/>
       <c r="AE15" s="1"/>
       <c r="AF15" s="39"/>
-      <c r="AH15" s="75"/>
+      <c r="AH15" s="68"/>
       <c r="AI15" s="1"/>
       <c r="AJ15" s="1"/>
       <c r="AK15" s="1"/>
-      <c r="AL15" s="69"/>
+      <c r="AL15" s="65"/>
       <c r="AM15" s="1"/>
       <c r="AN15" s="39"/>
     </row>
-    <row r="16" spans="1:40" ht="18" x14ac:dyDescent="0.55000000000000004">
+    <row r="16" spans="1:40" ht="19" x14ac:dyDescent="0.25">
       <c r="B16" s="15"/>
       <c r="C16" s="1"/>
-      <c r="H16" s="67"/>
+      <c r="H16" s="63"/>
       <c r="J16" s="15"/>
       <c r="K16" s="1"/>
-      <c r="P16" s="67"/>
+      <c r="P16" s="63"/>
       <c r="R16" s="15"/>
       <c r="S16" s="1"/>
-      <c r="X16" s="67"/>
-      <c r="Z16" s="75"/>
+      <c r="X16" s="63"/>
+      <c r="Z16" s="68"/>
       <c r="AA16" s="1"/>
       <c r="AB16" s="1"/>
-      <c r="AF16" s="67"/>
-      <c r="AH16" s="75"/>
+      <c r="AF16" s="63"/>
+      <c r="AH16" s="68"/>
       <c r="AI16" s="1"/>
       <c r="AJ16" s="1"/>
-      <c r="AN16" s="67"/>
+      <c r="AN16" s="63"/>
     </row>
-    <row r="17" spans="2:40" ht="18" x14ac:dyDescent="0.55000000000000004">
+    <row r="17" spans="2:40" ht="19" x14ac:dyDescent="0.25">
       <c r="B17" s="15"/>
       <c r="C17" s="1"/>
-      <c r="H17" s="67"/>
+      <c r="H17" s="63"/>
       <c r="J17" s="15"/>
       <c r="K17" s="1"/>
-      <c r="P17" s="67"/>
+      <c r="P17" s="63"/>
       <c r="R17" s="15"/>
       <c r="S17" s="1"/>
-      <c r="X17" s="67"/>
-      <c r="Z17" s="75"/>
+      <c r="X17" s="63"/>
+      <c r="Z17" s="68"/>
       <c r="AA17" s="1"/>
       <c r="AB17" s="1"/>
-      <c r="AF17" s="67"/>
-      <c r="AH17" s="75"/>
+      <c r="AF17" s="63"/>
+      <c r="AH17" s="68"/>
       <c r="AI17" s="1"/>
       <c r="AJ17" s="1"/>
-      <c r="AN17" s="67"/>
+      <c r="AN17" s="63"/>
     </row>
-    <row r="18" spans="2:40" ht="18" x14ac:dyDescent="0.55000000000000004">
+    <row r="18" spans="2:40" ht="19" x14ac:dyDescent="0.25">
       <c r="B18" s="15"/>
       <c r="C18" s="1"/>
       <c r="D18" s="2"/>
       <c r="E18" s="2"/>
       <c r="F18" s="2"/>
       <c r="G18" s="2"/>
-      <c r="H18" s="67"/>
+      <c r="H18" s="63"/>
       <c r="J18" s="15"/>
       <c r="K18" s="1"/>
       <c r="L18" s="2"/>
       <c r="M18" s="2"/>
       <c r="N18" s="2"/>
       <c r="O18" s="2"/>
-      <c r="P18" s="67"/>
+      <c r="P18" s="63"/>
       <c r="R18" s="15"/>
       <c r="S18" s="1"/>
       <c r="T18" s="2"/>
       <c r="U18" s="2"/>
       <c r="V18" s="2"/>
       <c r="W18" s="2"/>
-      <c r="X18" s="67"/>
-      <c r="Z18" s="75"/>
+      <c r="X18" s="63"/>
+      <c r="Z18" s="68"/>
       <c r="AA18" s="1"/>
       <c r="AB18" s="1"/>
-      <c r="AF18" s="67"/>
-      <c r="AH18" s="75"/>
+      <c r="AF18" s="63"/>
+      <c r="AH18" s="68"/>
       <c r="AI18" s="1"/>
       <c r="AJ18" s="1"/>
-      <c r="AN18" s="67"/>
+      <c r="AN18" s="63"/>
     </row>
-    <row r="19" spans="2:40" ht="18.399999999999999" thickBot="1" x14ac:dyDescent="0.6">
+    <row r="19" spans="2:40" ht="20" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B19" s="11"/>
       <c r="C19" s="12"/>
-      <c r="D19" s="79"/>
-      <c r="E19" s="79"/>
-      <c r="F19" s="79"/>
-      <c r="G19" s="79"/>
-      <c r="H19" s="78"/>
+      <c r="D19" s="72"/>
+      <c r="E19" s="72"/>
+      <c r="F19" s="72"/>
+      <c r="G19" s="72"/>
+      <c r="H19" s="71"/>
       <c r="J19" s="11"/>
       <c r="K19" s="12"/>
-      <c r="L19" s="79"/>
-      <c r="M19" s="79"/>
-      <c r="N19" s="79"/>
-      <c r="O19" s="79"/>
-      <c r="P19" s="78"/>
+      <c r="L19" s="72"/>
+      <c r="M19" s="72"/>
+      <c r="N19" s="72"/>
+      <c r="O19" s="72"/>
+      <c r="P19" s="71"/>
       <c r="R19" s="11"/>
       <c r="S19" s="12"/>
-      <c r="T19" s="79"/>
-      <c r="U19" s="79"/>
-      <c r="V19" s="79"/>
-      <c r="W19" s="79"/>
-      <c r="X19" s="78"/>
-      <c r="Z19" s="75"/>
+      <c r="T19" s="72"/>
+      <c r="U19" s="72"/>
+      <c r="V19" s="72"/>
+      <c r="W19" s="72"/>
+      <c r="X19" s="71"/>
+      <c r="Z19" s="68"/>
       <c r="AA19" s="2"/>
       <c r="AB19" s="1"/>
       <c r="AC19" s="2"/>
       <c r="AD19" s="2"/>
       <c r="AE19" s="2"/>
       <c r="AF19" s="40"/>
-      <c r="AH19" s="75"/>
+      <c r="AH19" s="68"/>
       <c r="AI19" s="2"/>
       <c r="AJ19" s="1"/>
       <c r="AK19" s="2"/>
@@ -43585,21 +43582,21 @@
       <c r="AM19" s="2"/>
       <c r="AN19" s="40"/>
     </row>
-    <row r="20" spans="2:40" ht="18.399999999999999" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="Z20" s="80"/>
-      <c r="AA20" s="79"/>
+    <row r="20" spans="2:40" ht="20" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="Z20" s="73"/>
+      <c r="AA20" s="72"/>
       <c r="AB20" s="12"/>
-      <c r="AC20" s="79"/>
-      <c r="AD20" s="79"/>
-      <c r="AE20" s="79"/>
-      <c r="AF20" s="78"/>
-      <c r="AH20" s="80"/>
-      <c r="AI20" s="79"/>
+      <c r="AC20" s="72"/>
+      <c r="AD20" s="72"/>
+      <c r="AE20" s="72"/>
+      <c r="AF20" s="71"/>
+      <c r="AH20" s="73"/>
+      <c r="AI20" s="72"/>
       <c r="AJ20" s="12"/>
-      <c r="AK20" s="79"/>
-      <c r="AL20" s="79"/>
-      <c r="AM20" s="79"/>
-      <c r="AN20" s="78"/>
+      <c r="AK20" s="72"/>
+      <c r="AL20" s="72"/>
+      <c r="AM20" s="72"/>
+      <c r="AN20" s="71"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -43625,47 +43622,45 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C8F61EE-9F60-994E-8E14-0022BD1ADF0E}">
   <dimension ref="A1:AP21"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.5"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="11" style="63"/>
-    <col min="2" max="3" width="4.3125" style="63" customWidth="1"/>
-    <col min="4" max="4" width="4.1875" style="63" customWidth="1"/>
-    <col min="5" max="5" width="4.3125" style="63" customWidth="1"/>
-    <col min="6" max="6" width="4.5" style="63" customWidth="1"/>
-    <col min="7" max="8" width="4.6875" style="63" customWidth="1"/>
-    <col min="9" max="9" width="9.1875" style="63" customWidth="1"/>
-    <col min="10" max="10" width="4.8125" style="63" customWidth="1"/>
-    <col min="11" max="11" width="5" style="63" customWidth="1"/>
-    <col min="12" max="12" width="4.8125" style="63" customWidth="1"/>
-    <col min="13" max="13" width="5" style="63" customWidth="1"/>
-    <col min="14" max="14" width="4.8125" style="63" customWidth="1"/>
-    <col min="15" max="15" width="4.6875" style="63" customWidth="1"/>
-    <col min="16" max="16" width="4.8125" style="63" customWidth="1"/>
-    <col min="17" max="17" width="9.1875" style="63" customWidth="1"/>
-    <col min="18" max="18" width="4.8125" style="63" customWidth="1"/>
-    <col min="19" max="20" width="5" style="63" customWidth="1"/>
-    <col min="21" max="23" width="4.6875" style="63" customWidth="1"/>
-    <col min="24" max="24" width="4.8125" style="63" customWidth="1"/>
-    <col min="25" max="25" width="9.8125" style="63" customWidth="1"/>
-    <col min="26" max="26" width="5.1875" style="63" customWidth="1"/>
-    <col min="27" max="27" width="5" style="63" customWidth="1"/>
-    <col min="28" max="28" width="4.8125" style="63" customWidth="1"/>
-    <col min="29" max="29" width="4.6875" style="63" customWidth="1"/>
-    <col min="30" max="30" width="4.8125" style="63" customWidth="1"/>
-    <col min="31" max="32" width="5" style="63" customWidth="1"/>
-    <col min="33" max="33" width="4.8125" style="63" customWidth="1"/>
-    <col min="34" max="34" width="10.1875" style="63" customWidth="1"/>
-    <col min="35" max="35" width="4.8125" style="63" customWidth="1"/>
-    <col min="36" max="37" width="5.1875" style="63" customWidth="1"/>
-    <col min="38" max="38" width="5" style="63" customWidth="1"/>
-    <col min="39" max="39" width="4.8125" style="63" customWidth="1"/>
-    <col min="40" max="40" width="5" style="63" customWidth="1"/>
-    <col min="41" max="41" width="4.8125" style="63" customWidth="1"/>
-    <col min="42" max="42" width="4.6875" style="63" customWidth="1"/>
-    <col min="43" max="16384" width="11" style="63"/>
+    <col min="2" max="3" width="4.33203125" customWidth="1"/>
+    <col min="4" max="4" width="4.1640625" customWidth="1"/>
+    <col min="5" max="5" width="4.33203125" customWidth="1"/>
+    <col min="6" max="6" width="4.5" customWidth="1"/>
+    <col min="7" max="8" width="4.6640625" customWidth="1"/>
+    <col min="9" max="9" width="9.1640625" customWidth="1"/>
+    <col min="10" max="10" width="4.83203125" customWidth="1"/>
+    <col min="11" max="11" width="5" customWidth="1"/>
+    <col min="12" max="12" width="4.83203125" customWidth="1"/>
+    <col min="13" max="13" width="5" customWidth="1"/>
+    <col min="14" max="14" width="4.83203125" customWidth="1"/>
+    <col min="15" max="15" width="4.6640625" customWidth="1"/>
+    <col min="16" max="16" width="4.83203125" customWidth="1"/>
+    <col min="17" max="17" width="9.1640625" customWidth="1"/>
+    <col min="18" max="18" width="4.83203125" customWidth="1"/>
+    <col min="19" max="20" width="5" customWidth="1"/>
+    <col min="21" max="23" width="4.6640625" customWidth="1"/>
+    <col min="24" max="24" width="4.83203125" customWidth="1"/>
+    <col min="25" max="25" width="9.83203125" customWidth="1"/>
+    <col min="26" max="26" width="5.1640625" customWidth="1"/>
+    <col min="27" max="27" width="5" customWidth="1"/>
+    <col min="28" max="28" width="4.83203125" customWidth="1"/>
+    <col min="29" max="29" width="4.6640625" customWidth="1"/>
+    <col min="30" max="30" width="4.83203125" customWidth="1"/>
+    <col min="31" max="32" width="5" customWidth="1"/>
+    <col min="33" max="33" width="4.83203125" customWidth="1"/>
+    <col min="34" max="34" width="10.1640625" customWidth="1"/>
+    <col min="35" max="35" width="4.83203125" customWidth="1"/>
+    <col min="36" max="37" width="5.1640625" customWidth="1"/>
+    <col min="38" max="38" width="5" customWidth="1"/>
+    <col min="39" max="39" width="4.83203125" customWidth="1"/>
+    <col min="40" max="40" width="5" customWidth="1"/>
+    <col min="41" max="41" width="4.83203125" customWidth="1"/>
+    <col min="42" max="42" width="4.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:42" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:42" s="2" customFormat="1" ht="19" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>51</v>
       </c>
@@ -43684,12 +43679,12 @@
       <c r="O1" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="R1" s="81" t="s">
+      <c r="R1" s="74" t="s">
         <v>50</v>
       </c>
       <c r="S1" s="1"/>
     </row>
-    <row r="3" spans="1:42" ht="18.399999999999999" thickBot="1" x14ac:dyDescent="0.6">
+    <row r="3" spans="1:42" ht="20" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="2" t="str">
         <f>IF(ISBLANK(E10)=TRUE,"NOT DONE",IF(B5=E10,"CORRECT", "INCORRECT"))</f>
         <v>NOT DONE</v>
@@ -43738,56 +43733,56 @@
       <c r="AN3" s="2"/>
       <c r="AO3" s="2"/>
     </row>
-    <row r="4" spans="1:42" ht="18" x14ac:dyDescent="0.55000000000000004">
-      <c r="B4" s="64" t="s">
+    <row r="4" spans="1:42" ht="19" x14ac:dyDescent="0.25">
+      <c r="B4" s="80" t="s">
         <v>20</v>
       </c>
-      <c r="C4" s="65"/>
-      <c r="D4" s="65"/>
-      <c r="E4" s="65"/>
-      <c r="F4" s="65"/>
-      <c r="G4" s="65"/>
-      <c r="H4" s="66"/>
-      <c r="J4" s="64" t="s">
+      <c r="C4" s="81"/>
+      <c r="D4" s="81"/>
+      <c r="E4" s="81"/>
+      <c r="F4" s="81"/>
+      <c r="G4" s="81"/>
+      <c r="H4" s="82"/>
+      <c r="J4" s="80" t="s">
         <v>21</v>
       </c>
-      <c r="K4" s="65"/>
-      <c r="L4" s="65"/>
-      <c r="M4" s="65"/>
-      <c r="N4" s="65"/>
-      <c r="O4" s="65"/>
-      <c r="P4" s="66"/>
-      <c r="R4" s="64" t="s">
+      <c r="K4" s="81"/>
+      <c r="L4" s="81"/>
+      <c r="M4" s="81"/>
+      <c r="N4" s="81"/>
+      <c r="O4" s="81"/>
+      <c r="P4" s="82"/>
+      <c r="R4" s="80" t="s">
         <v>22</v>
       </c>
-      <c r="S4" s="65"/>
-      <c r="T4" s="65"/>
-      <c r="U4" s="65"/>
-      <c r="V4" s="65"/>
-      <c r="W4" s="65"/>
-      <c r="X4" s="66"/>
-      <c r="Z4" s="64" t="s">
+      <c r="S4" s="81"/>
+      <c r="T4" s="81"/>
+      <c r="U4" s="81"/>
+      <c r="V4" s="81"/>
+      <c r="W4" s="81"/>
+      <c r="X4" s="82"/>
+      <c r="Z4" s="80" t="s">
         <v>23</v>
       </c>
-      <c r="AA4" s="65"/>
-      <c r="AB4" s="65"/>
-      <c r="AC4" s="65"/>
-      <c r="AD4" s="65"/>
-      <c r="AE4" s="65"/>
-      <c r="AF4" s="65"/>
-      <c r="AG4" s="66"/>
-      <c r="AI4" s="64" t="s">
+      <c r="AA4" s="81"/>
+      <c r="AB4" s="81"/>
+      <c r="AC4" s="81"/>
+      <c r="AD4" s="81"/>
+      <c r="AE4" s="81"/>
+      <c r="AF4" s="81"/>
+      <c r="AG4" s="82"/>
+      <c r="AI4" s="80" t="s">
         <v>24</v>
       </c>
-      <c r="AJ4" s="65"/>
-      <c r="AK4" s="65"/>
-      <c r="AL4" s="65"/>
-      <c r="AM4" s="65"/>
-      <c r="AN4" s="65"/>
-      <c r="AO4" s="65"/>
-      <c r="AP4" s="66"/>
+      <c r="AJ4" s="81"/>
+      <c r="AK4" s="81"/>
+      <c r="AL4" s="81"/>
+      <c r="AM4" s="81"/>
+      <c r="AN4" s="81"/>
+      <c r="AO4" s="81"/>
+      <c r="AP4" s="82"/>
     </row>
-    <row r="5" spans="1:42" ht="18" x14ac:dyDescent="0.55000000000000004">
+    <row r="5" spans="1:42" ht="19" x14ac:dyDescent="0.25">
       <c r="B5" s="9">
         <f>G10-G6*C10-G7*D10</f>
         <v>5</v>
@@ -43797,7 +43792,7 @@
       <c r="E5" s="2"/>
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
-      <c r="H5" s="67"/>
+      <c r="H5" s="63"/>
       <c r="J5" s="9">
         <f>(O10-M10-O7*L10)/O6</f>
         <v>2</v>
@@ -43807,7 +43802,7 @@
       <c r="M5" s="2"/>
       <c r="N5" s="2"/>
       <c r="O5" s="2"/>
-      <c r="P5" s="67"/>
+      <c r="P5" s="63"/>
       <c r="R5" s="9">
         <f>(W11-U11-T11*W7)/W6</f>
         <v>3</v>
@@ -43817,7 +43812,7 @@
       <c r="U5" s="2"/>
       <c r="V5" s="2"/>
       <c r="W5" s="2"/>
-      <c r="X5" s="67"/>
+      <c r="X5" s="63"/>
       <c r="Z5" s="9">
         <f>(AF11-AD11-AA11*AF6-AB11*AF7)/AF8</f>
         <v>-1</v>
@@ -43828,7 +43823,7 @@
       <c r="AD5" s="2"/>
       <c r="AE5" s="2"/>
       <c r="AF5" s="2"/>
-      <c r="AG5" s="67"/>
+      <c r="AG5" s="63"/>
       <c r="AI5" s="9">
         <f>AO12-AJ12*AO6-AK12*AO7-AL12*AO8</f>
         <v>-4</v>
@@ -43839,9 +43834,9 @@
       <c r="AM5" s="2"/>
       <c r="AN5" s="2"/>
       <c r="AO5" s="2"/>
-      <c r="AP5" s="67"/>
+      <c r="AP5" s="63"/>
     </row>
-    <row r="6" spans="1:42" ht="21" x14ac:dyDescent="0.55000000000000004">
+    <row r="6" spans="1:42" ht="19" x14ac:dyDescent="0.25">
       <c r="B6" s="10"/>
       <c r="C6" s="2"/>
       <c r="D6" s="1"/>
@@ -43850,7 +43845,7 @@
       <c r="G6" s="29">
         <v>3</v>
       </c>
-      <c r="H6" s="70" t="s">
+      <c r="H6" s="66" t="s">
         <v>55</v>
       </c>
       <c r="J6" s="10"/>
@@ -43861,7 +43856,7 @@
       <c r="O6" s="29">
         <v>3</v>
       </c>
-      <c r="P6" s="70" t="s">
+      <c r="P6" s="66" t="s">
         <v>55</v>
       </c>
       <c r="R6" s="10"/>
@@ -43872,7 +43867,7 @@
       <c r="W6" s="29">
         <v>2</v>
       </c>
-      <c r="X6" s="70" t="s">
+      <c r="X6" s="66" t="s">
         <v>55</v>
       </c>
       <c r="Z6" s="10"/>
@@ -43884,7 +43879,7 @@
       <c r="AF6" s="29">
         <v>2</v>
       </c>
-      <c r="AG6" s="70" t="s">
+      <c r="AG6" s="66" t="s">
         <v>55</v>
       </c>
       <c r="AI6" s="10"/>
@@ -43896,11 +43891,11 @@
       <c r="AO6" s="29">
         <v>2</v>
       </c>
-      <c r="AP6" s="70" t="s">
+      <c r="AP6" s="66" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="7" spans="1:42" ht="21" x14ac:dyDescent="0.55000000000000004">
+    <row r="7" spans="1:42" ht="19" x14ac:dyDescent="0.25">
       <c r="B7" s="10"/>
       <c r="C7" s="2"/>
       <c r="D7" s="1"/>
@@ -43909,7 +43904,7 @@
       <c r="G7" s="29">
         <v>2</v>
       </c>
-      <c r="H7" s="70" t="s">
+      <c r="H7" s="66" t="s">
         <v>56</v>
       </c>
       <c r="J7" s="10"/>
@@ -43920,7 +43915,7 @@
       <c r="O7" s="29">
         <v>2</v>
       </c>
-      <c r="P7" s="70" t="s">
+      <c r="P7" s="66" t="s">
         <v>56</v>
       </c>
       <c r="R7" s="10"/>
@@ -43931,7 +43926,7 @@
       <c r="W7" s="29">
         <v>1</v>
       </c>
-      <c r="X7" s="70" t="s">
+      <c r="X7" s="66" t="s">
         <v>56</v>
       </c>
       <c r="Z7" s="10"/>
@@ -43943,7 +43938,7 @@
       <c r="AF7" s="29">
         <v>1</v>
       </c>
-      <c r="AG7" s="70" t="s">
+      <c r="AG7" s="66" t="s">
         <v>56</v>
       </c>
       <c r="AI7" s="10"/>
@@ -43955,16 +43950,16 @@
       <c r="AO7" s="29">
         <v>5</v>
       </c>
-      <c r="AP7" s="70" t="s">
+      <c r="AP7" s="66" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="8" spans="1:42" ht="21.4" thickBot="1" x14ac:dyDescent="0.6">
+    <row r="8" spans="1:42" ht="20" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B8" s="10"/>
-      <c r="C8" s="82" t="s">
+      <c r="C8" s="86" t="s">
         <v>47</v>
       </c>
-      <c r="D8" s="82"/>
+      <c r="D8" s="86"/>
       <c r="E8" s="47" t="s">
         <v>48</v>
       </c>
@@ -43972,12 +43967,12 @@
       <c r="G8" s="17">
         <v>1</v>
       </c>
-      <c r="H8" s="68"/>
+      <c r="H8" s="64"/>
       <c r="J8" s="10"/>
-      <c r="K8" s="82" t="s">
+      <c r="K8" s="86" t="s">
         <v>47</v>
       </c>
-      <c r="L8" s="82"/>
+      <c r="L8" s="86"/>
       <c r="M8" s="47" t="s">
         <v>48</v>
       </c>
@@ -43985,12 +43980,12 @@
       <c r="O8" s="17">
         <v>1</v>
       </c>
-      <c r="P8" s="68"/>
+      <c r="P8" s="64"/>
       <c r="R8" s="10"/>
-      <c r="S8" s="82" t="s">
+      <c r="S8" s="86" t="s">
         <v>47</v>
       </c>
-      <c r="T8" s="82"/>
+      <c r="T8" s="86"/>
       <c r="U8" s="47" t="s">
         <v>48</v>
       </c>
@@ -43998,33 +43993,33 @@
       <c r="W8" s="17">
         <v>1</v>
       </c>
-      <c r="X8" s="68"/>
-      <c r="Z8" s="86"/>
-      <c r="AA8" s="85"/>
-      <c r="AB8" s="85"/>
-      <c r="AC8" s="85"/>
-      <c r="AD8" s="85"/>
-      <c r="AE8" s="85"/>
+      <c r="X8" s="64"/>
+      <c r="Z8" s="78"/>
+      <c r="AA8" s="77"/>
+      <c r="AB8" s="77"/>
+      <c r="AC8" s="77"/>
+      <c r="AD8" s="77"/>
+      <c r="AE8" s="77"/>
       <c r="AF8" s="29">
         <v>2</v>
       </c>
-      <c r="AG8" s="87" t="s">
+      <c r="AG8" s="79" t="s">
         <v>57</v>
       </c>
-      <c r="AI8" s="86"/>
-      <c r="AJ8" s="85"/>
-      <c r="AK8" s="85"/>
-      <c r="AL8" s="85"/>
-      <c r="AM8" s="85"/>
-      <c r="AN8" s="85"/>
+      <c r="AI8" s="78"/>
+      <c r="AJ8" s="77"/>
+      <c r="AK8" s="77"/>
+      <c r="AL8" s="77"/>
+      <c r="AM8" s="77"/>
+      <c r="AN8" s="77"/>
       <c r="AO8" s="29">
         <v>1</v>
       </c>
-      <c r="AP8" s="87" t="s">
+      <c r="AP8" s="79" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="9" spans="1:42" ht="21.4" thickBot="1" x14ac:dyDescent="0.6">
+    <row r="9" spans="1:42" ht="20" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B9" s="10"/>
       <c r="C9" s="20">
         <v>1</v>
@@ -44042,7 +44037,7 @@
         <f>C9*G6+D9*G7+E9</f>
         <v>8</v>
       </c>
-      <c r="H9" s="71" t="s">
+      <c r="H9" s="67" t="s">
         <v>52</v>
       </c>
       <c r="J9" s="10"/>
@@ -44062,7 +44057,7 @@
         <f>K9*O6+L9*O7+M9</f>
         <v>5</v>
       </c>
-      <c r="P9" s="71" t="s">
+      <c r="P9" s="67" t="s">
         <v>52</v>
       </c>
       <c r="R9" s="10"/>
@@ -44082,15 +44077,15 @@
         <f>S9*W6+T9*W7+U9</f>
         <v>3</v>
       </c>
-      <c r="X9" s="71" t="s">
+      <c r="X9" s="67" t="s">
         <v>52</v>
       </c>
       <c r="Z9" s="46"/>
-      <c r="AA9" s="88" t="s">
+      <c r="AA9" s="87" t="s">
         <v>47</v>
       </c>
-      <c r="AB9" s="88"/>
-      <c r="AC9" s="88"/>
+      <c r="AB9" s="87"/>
+      <c r="AC9" s="87"/>
       <c r="AD9" s="47" t="s">
         <v>48</v>
       </c>
@@ -44098,13 +44093,13 @@
       <c r="AF9" s="45">
         <v>1</v>
       </c>
-      <c r="AG9" s="68"/>
+      <c r="AG9" s="64"/>
       <c r="AI9" s="46"/>
-      <c r="AJ9" s="88" t="s">
+      <c r="AJ9" s="87" t="s">
         <v>47</v>
       </c>
-      <c r="AK9" s="88"/>
-      <c r="AL9" s="88"/>
+      <c r="AK9" s="87"/>
+      <c r="AL9" s="87"/>
       <c r="AM9" s="47" t="s">
         <v>48</v>
       </c>
@@ -44112,10 +44107,10 @@
       <c r="AO9" s="45">
         <v>1</v>
       </c>
-      <c r="AP9" s="68"/>
+      <c r="AP9" s="64"/>
     </row>
-    <row r="10" spans="1:42" ht="21.4" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="B10" s="75"/>
+    <row r="10" spans="1:42" ht="20" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B10" s="68"/>
       <c r="C10" s="34">
         <v>1</v>
       </c>
@@ -44129,10 +44124,10 @@
       <c r="G10" s="44">
         <v>12</v>
       </c>
-      <c r="H10" s="71" t="s">
+      <c r="H10" s="67" t="s">
         <v>53</v>
       </c>
-      <c r="J10" s="75"/>
+      <c r="J10" s="68"/>
       <c r="K10" s="58"/>
       <c r="L10" s="16">
         <v>1</v>
@@ -44146,10 +44141,10 @@
       <c r="O10" s="42">
         <v>8</v>
       </c>
-      <c r="P10" s="71" t="s">
+      <c r="P10" s="67" t="s">
         <v>53</v>
       </c>
-      <c r="R10" s="75"/>
+      <c r="R10" s="68"/>
       <c r="S10" s="25">
         <v>2</v>
       </c>
@@ -44166,7 +44161,7 @@
         <f>S10*W6+T10*W7+U10</f>
         <v>5</v>
       </c>
-      <c r="X10" s="71" t="s">
+      <c r="X10" s="67" t="s">
         <v>53</v>
       </c>
       <c r="Z10" s="10"/>
@@ -44189,7 +44184,7 @@
         <f>AA10*AF6+AB10*AF7+AC10*AF8+AD10</f>
         <v>3</v>
       </c>
-      <c r="AG10" s="71" t="s">
+      <c r="AG10" s="67" t="s">
         <v>52</v>
       </c>
       <c r="AI10" s="10"/>
@@ -44212,14 +44207,14 @@
         <f>AJ10*AO6+AK10*AO7+AL10*AO8+AM10</f>
         <v>7</v>
       </c>
-      <c r="AP10" s="71" t="s">
+      <c r="AP10" s="67" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="11" spans="1:42" ht="21.4" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="B11" s="76"/>
-      <c r="H11" s="77"/>
-      <c r="J11" s="76"/>
+    <row r="11" spans="1:42" ht="20" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B11" s="69"/>
+      <c r="H11" s="70"/>
+      <c r="J11" s="69"/>
       <c r="K11" s="34">
         <v>3</v>
       </c>
@@ -44236,10 +44231,10 @@
         <f>K11*O6+O7*L11+M11</f>
         <v>9</v>
       </c>
-      <c r="P11" s="71" t="s">
+      <c r="P11" s="67" t="s">
         <v>54</v>
       </c>
-      <c r="R11" s="76"/>
+      <c r="R11" s="69"/>
       <c r="S11" s="59"/>
       <c r="T11" s="35">
         <v>1</v>
@@ -44253,10 +44248,10 @@
       <c r="W11" s="16">
         <v>7</v>
       </c>
-      <c r="X11" s="71" t="s">
+      <c r="X11" s="67" t="s">
         <v>54</v>
       </c>
-      <c r="Z11" s="75"/>
+      <c r="Z11" s="68"/>
       <c r="AA11" s="48">
         <v>1</v>
       </c>
@@ -44273,10 +44268,10 @@
       <c r="AF11" s="60">
         <v>1</v>
       </c>
-      <c r="AG11" s="71" t="s">
+      <c r="AG11" s="67" t="s">
         <v>53</v>
       </c>
-      <c r="AI11" s="75"/>
+      <c r="AI11" s="68"/>
       <c r="AJ11" s="48">
         <v>1</v>
       </c>
@@ -44296,23 +44291,23 @@
         <f>AJ11*AO6+AK11*AO7+AL11*AO8+AM11</f>
         <v>5</v>
       </c>
-      <c r="AP11" s="71" t="s">
+      <c r="AP11" s="67" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="12" spans="1:42" ht="21.4" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="B12" s="75"/>
+    <row r="12" spans="1:42" ht="20" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B12" s="68"/>
       <c r="C12" s="1"/>
-      <c r="D12" s="83"/>
+      <c r="D12" s="75"/>
       <c r="E12" s="1"/>
-      <c r="F12" s="69"/>
+      <c r="F12" s="65"/>
       <c r="G12" s="1"/>
       <c r="H12" s="39"/>
-      <c r="J12" s="75"/>
-      <c r="P12" s="67"/>
-      <c r="R12" s="75"/>
-      <c r="X12" s="67"/>
-      <c r="Z12" s="75"/>
+      <c r="J12" s="68"/>
+      <c r="P12" s="63"/>
+      <c r="R12" s="68"/>
+      <c r="X12" s="63"/>
+      <c r="Z12" s="68"/>
       <c r="AA12" s="34">
         <v>1</v>
       </c>
@@ -44332,10 +44327,10 @@
         <f>AA12*AF6+AB12*AF7+AC12*AF8+AD12</f>
         <v>5</v>
       </c>
-      <c r="AG12" s="71" t="s">
+      <c r="AG12" s="67" t="s">
         <v>54</v>
       </c>
-      <c r="AI12" s="75"/>
+      <c r="AI12" s="68"/>
       <c r="AJ12" s="34">
         <v>1</v>
       </c>
@@ -44352,181 +44347,181 @@
       <c r="AO12" s="16">
         <v>3</v>
       </c>
-      <c r="AP12" s="71" t="s">
+      <c r="AP12" s="67" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="13" spans="1:42" ht="18" x14ac:dyDescent="0.55000000000000004">
-      <c r="B13" s="75"/>
+    <row r="13" spans="1:42" ht="19" x14ac:dyDescent="0.25">
+      <c r="B13" s="68"/>
       <c r="C13" s="1"/>
       <c r="D13" s="1"/>
       <c r="E13" s="1"/>
-      <c r="F13" s="69"/>
+      <c r="F13" s="65"/>
       <c r="G13" s="1"/>
       <c r="H13" s="39"/>
-      <c r="J13" s="75"/>
+      <c r="J13" s="68"/>
       <c r="P13" s="39"/>
-      <c r="R13" s="75"/>
+      <c r="R13" s="68"/>
       <c r="X13" s="39"/>
-      <c r="Z13" s="75"/>
-      <c r="AG13" s="67"/>
-      <c r="AI13" s="75"/>
-      <c r="AP13" s="67"/>
+      <c r="Z13" s="68"/>
+      <c r="AG13" s="63"/>
+      <c r="AI13" s="68"/>
+      <c r="AP13" s="63"/>
     </row>
-    <row r="14" spans="1:42" ht="18" x14ac:dyDescent="0.55000000000000004">
-      <c r="B14" s="75"/>
+    <row r="14" spans="1:42" ht="19" x14ac:dyDescent="0.25">
+      <c r="B14" s="68"/>
       <c r="C14" s="1"/>
       <c r="D14" s="1"/>
       <c r="E14" s="1"/>
-      <c r="F14" s="69"/>
+      <c r="F14" s="65"/>
       <c r="G14" s="1"/>
       <c r="H14" s="39"/>
-      <c r="J14" s="75"/>
+      <c r="J14" s="68"/>
       <c r="P14" s="39"/>
-      <c r="R14" s="75"/>
+      <c r="R14" s="68"/>
       <c r="X14" s="39"/>
-      <c r="Z14" s="75"/>
-      <c r="AG14" s="67"/>
-      <c r="AI14" s="75"/>
-      <c r="AP14" s="67"/>
+      <c r="Z14" s="68"/>
+      <c r="AG14" s="63"/>
+      <c r="AI14" s="68"/>
+      <c r="AP14" s="63"/>
     </row>
-    <row r="15" spans="1:42" ht="18" x14ac:dyDescent="0.55000000000000004">
-      <c r="B15" s="75"/>
+    <row r="15" spans="1:42" ht="19" x14ac:dyDescent="0.25">
+      <c r="B15" s="68"/>
       <c r="C15" s="1"/>
       <c r="D15" s="1"/>
       <c r="E15" s="1"/>
-      <c r="F15" s="69"/>
+      <c r="F15" s="65"/>
       <c r="G15" s="1"/>
       <c r="H15" s="39"/>
-      <c r="J15" s="75"/>
+      <c r="J15" s="68"/>
       <c r="P15" s="39"/>
-      <c r="R15" s="75"/>
+      <c r="R15" s="68"/>
       <c r="X15" s="39"/>
-      <c r="Z15" s="75"/>
-      <c r="AG15" s="67"/>
-      <c r="AI15" s="75"/>
-      <c r="AP15" s="67"/>
+      <c r="Z15" s="68"/>
+      <c r="AG15" s="63"/>
+      <c r="AI15" s="68"/>
+      <c r="AP15" s="63"/>
     </row>
-    <row r="16" spans="1:42" ht="18" x14ac:dyDescent="0.55000000000000004">
-      <c r="B16" s="75"/>
+    <row r="16" spans="1:42" ht="19" x14ac:dyDescent="0.25">
+      <c r="B16" s="68"/>
       <c r="C16" s="1"/>
       <c r="D16" s="1"/>
-      <c r="H16" s="67"/>
-      <c r="J16" s="75"/>
+      <c r="H16" s="63"/>
+      <c r="J16" s="68"/>
       <c r="P16" s="39"/>
-      <c r="R16" s="75"/>
+      <c r="R16" s="68"/>
       <c r="X16" s="39"/>
-      <c r="Z16" s="75"/>
-      <c r="AG16" s="67"/>
-      <c r="AI16" s="75"/>
-      <c r="AP16" s="67"/>
+      <c r="Z16" s="68"/>
+      <c r="AG16" s="63"/>
+      <c r="AI16" s="68"/>
+      <c r="AP16" s="63"/>
     </row>
-    <row r="17" spans="2:42" ht="18" x14ac:dyDescent="0.55000000000000004">
-      <c r="B17" s="75"/>
+    <row r="17" spans="2:42" ht="19" x14ac:dyDescent="0.25">
+      <c r="B17" s="68"/>
       <c r="C17" s="1"/>
       <c r="D17" s="1"/>
-      <c r="H17" s="67"/>
-      <c r="J17" s="75"/>
-      <c r="P17" s="67"/>
-      <c r="R17" s="75"/>
-      <c r="X17" s="67"/>
-      <c r="Z17" s="75"/>
-      <c r="AG17" s="67"/>
-      <c r="AI17" s="75"/>
-      <c r="AP17" s="67"/>
+      <c r="H17" s="63"/>
+      <c r="J17" s="68"/>
+      <c r="P17" s="63"/>
+      <c r="R17" s="68"/>
+      <c r="X17" s="63"/>
+      <c r="Z17" s="68"/>
+      <c r="AG17" s="63"/>
+      <c r="AI17" s="68"/>
+      <c r="AP17" s="63"/>
     </row>
-    <row r="18" spans="2:42" ht="18" x14ac:dyDescent="0.55000000000000004">
-      <c r="B18" s="75"/>
+    <row r="18" spans="2:42" ht="19" x14ac:dyDescent="0.25">
+      <c r="B18" s="68"/>
       <c r="C18" s="1"/>
       <c r="D18" s="1"/>
-      <c r="H18" s="67"/>
-      <c r="J18" s="75"/>
-      <c r="P18" s="67"/>
-      <c r="R18" s="75"/>
-      <c r="X18" s="67"/>
-      <c r="Z18" s="75"/>
-      <c r="AG18" s="67"/>
-      <c r="AI18" s="75"/>
-      <c r="AP18" s="67"/>
+      <c r="H18" s="63"/>
+      <c r="J18" s="68"/>
+      <c r="P18" s="63"/>
+      <c r="R18" s="68"/>
+      <c r="X18" s="63"/>
+      <c r="Z18" s="68"/>
+      <c r="AG18" s="63"/>
+      <c r="AI18" s="68"/>
+      <c r="AP18" s="63"/>
     </row>
-    <row r="19" spans="2:42" ht="18" x14ac:dyDescent="0.55000000000000004">
-      <c r="B19" s="75"/>
+    <row r="19" spans="2:42" ht="19" x14ac:dyDescent="0.25">
+      <c r="B19" s="68"/>
       <c r="C19" s="2"/>
       <c r="D19" s="1"/>
       <c r="E19" s="2"/>
       <c r="F19" s="2"/>
       <c r="G19" s="2"/>
       <c r="H19" s="40"/>
-      <c r="J19" s="75"/>
-      <c r="P19" s="67"/>
-      <c r="R19" s="75"/>
-      <c r="X19" s="67"/>
-      <c r="Z19" s="75"/>
-      <c r="AG19" s="67"/>
-      <c r="AI19" s="75"/>
-      <c r="AP19" s="67"/>
+      <c r="J19" s="68"/>
+      <c r="P19" s="63"/>
+      <c r="R19" s="68"/>
+      <c r="X19" s="63"/>
+      <c r="Z19" s="68"/>
+      <c r="AG19" s="63"/>
+      <c r="AI19" s="68"/>
+      <c r="AP19" s="63"/>
     </row>
-    <row r="20" spans="2:42" ht="18.399999999999999" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="B20" s="80"/>
-      <c r="C20" s="79"/>
+    <row r="20" spans="2:42" ht="20" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B20" s="73"/>
+      <c r="C20" s="72"/>
       <c r="D20" s="12"/>
-      <c r="E20" s="79"/>
-      <c r="F20" s="79"/>
-      <c r="G20" s="79"/>
-      <c r="H20" s="78"/>
-      <c r="J20" s="75"/>
+      <c r="E20" s="72"/>
+      <c r="F20" s="72"/>
+      <c r="G20" s="72"/>
+      <c r="H20" s="71"/>
+      <c r="J20" s="68"/>
       <c r="P20" s="40"/>
-      <c r="R20" s="75"/>
+      <c r="R20" s="68"/>
       <c r="X20" s="40"/>
-      <c r="Z20" s="75"/>
-      <c r="AG20" s="67"/>
-      <c r="AI20" s="75"/>
-      <c r="AP20" s="67"/>
+      <c r="Z20" s="68"/>
+      <c r="AG20" s="63"/>
+      <c r="AI20" s="68"/>
+      <c r="AP20" s="63"/>
     </row>
-    <row r="21" spans="2:42" ht="16.149999999999999" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="J21" s="80"/>
-      <c r="K21" s="79"/>
-      <c r="L21" s="79"/>
-      <c r="M21" s="79"/>
-      <c r="N21" s="79"/>
-      <c r="O21" s="79"/>
-      <c r="P21" s="78"/>
-      <c r="R21" s="80"/>
-      <c r="S21" s="79"/>
-      <c r="T21" s="79"/>
-      <c r="U21" s="79"/>
-      <c r="V21" s="79"/>
-      <c r="W21" s="79"/>
-      <c r="X21" s="78"/>
-      <c r="Z21" s="80"/>
-      <c r="AA21" s="79"/>
-      <c r="AB21" s="79"/>
-      <c r="AC21" s="79"/>
-      <c r="AD21" s="79"/>
-      <c r="AE21" s="79"/>
-      <c r="AF21" s="79"/>
-      <c r="AG21" s="78"/>
-      <c r="AI21" s="80"/>
-      <c r="AJ21" s="79"/>
-      <c r="AK21" s="79"/>
-      <c r="AL21" s="79"/>
-      <c r="AM21" s="79"/>
-      <c r="AN21" s="79"/>
-      <c r="AO21" s="79"/>
-      <c r="AP21" s="78"/>
+    <row r="21" spans="2:42" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="J21" s="73"/>
+      <c r="K21" s="72"/>
+      <c r="L21" s="72"/>
+      <c r="M21" s="72"/>
+      <c r="N21" s="72"/>
+      <c r="O21" s="72"/>
+      <c r="P21" s="71"/>
+      <c r="R21" s="73"/>
+      <c r="S21" s="72"/>
+      <c r="T21" s="72"/>
+      <c r="U21" s="72"/>
+      <c r="V21" s="72"/>
+      <c r="W21" s="72"/>
+      <c r="X21" s="71"/>
+      <c r="Z21" s="73"/>
+      <c r="AA21" s="72"/>
+      <c r="AB21" s="72"/>
+      <c r="AC21" s="72"/>
+      <c r="AD21" s="72"/>
+      <c r="AE21" s="72"/>
+      <c r="AF21" s="72"/>
+      <c r="AG21" s="71"/>
+      <c r="AI21" s="73"/>
+      <c r="AJ21" s="72"/>
+      <c r="AK21" s="72"/>
+      <c r="AL21" s="72"/>
+      <c r="AM21" s="72"/>
+      <c r="AN21" s="72"/>
+      <c r="AO21" s="72"/>
+      <c r="AP21" s="71"/>
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="Z4:AG4"/>
+    <mergeCell ref="AA9:AC9"/>
+    <mergeCell ref="AI4:AP4"/>
+    <mergeCell ref="AJ9:AL9"/>
     <mergeCell ref="B4:H4"/>
     <mergeCell ref="C8:D8"/>
     <mergeCell ref="J4:P4"/>
     <mergeCell ref="K8:L8"/>
     <mergeCell ref="R4:X4"/>
     <mergeCell ref="S8:T8"/>
-    <mergeCell ref="Z4:AG4"/>
-    <mergeCell ref="AA9:AC9"/>
-    <mergeCell ref="AI4:AP4"/>
-    <mergeCell ref="AJ9:AL9"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="R1" r:id="rId1" xr:uid="{45024357-32C1-ED48-9305-5D55817EC8E5}"/>
@@ -44539,112 +44534,112 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C0963377-E106-E649-9375-6D590D9A623A}">
   <dimension ref="A1:A23"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.5"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="92" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.5">
+    <row r="1" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A1" s="3" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.5">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A2" s="3"/>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.5">
+    <row r="3" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.5">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A4" s="3"/>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.5">
+    <row r="5" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.5">
+    <row r="6" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A6" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.5">
+    <row r="7" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A7" s="3" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.5">
+    <row r="8" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A8" s="3" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.5">
+    <row r="9" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A9" s="3" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.5">
+    <row r="10" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A10" s="3" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.5">
+    <row r="11" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A11" s="4"/>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.5">
+    <row r="12" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A12" s="3" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.5">
+    <row r="13" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A13" s="3" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.5">
+    <row r="14" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A14" s="3"/>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.5">
+    <row r="15" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A15" s="3" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.5">
+    <row r="16" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A16" s="3" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.5">
+    <row r="17" spans="1:1" ht="34" x14ac:dyDescent="0.2">
       <c r="A17" s="3" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.5">
+    <row r="18" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A18" s="3" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.5">
+    <row r="19" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A19" s="3" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="20" spans="1:1" ht="30.75" x14ac:dyDescent="0.5">
+    <row r="20" spans="1:1" ht="34" x14ac:dyDescent="0.2">
       <c r="A20" s="3" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.5">
+    <row r="21" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A21" s="3" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.5">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A22" s="3"/>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.5">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A23" s="3"/>
     </row>
   </sheetData>

</xml_diff>